<commit_message>
Complete DBM form source mapping starter
- add verified printed-manual and PDF page ranges for all 31 DBM LGU form entries
- expand candidate field mappings from 25 representative rows to 70 source-anchored structures
- cover every listed LBP, LBA, LBR, LBE, and LBAc form without asserting local applicability
- retain explicit control, ownership, print, signatory, and acceptance boundaries
- update the operator guide, canonical Finance roadmap, and changelog with the stronger evidence position
</commit_message>
<xml_diff>
--- a/outputs/grand-finance-field-acceptance/GRAND_Finance_Field_Acceptance_Starter.xlsx
+++ b/outputs/grand-finance-field-acceptance/GRAND_Finance_Field_Acceptance_Starter.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R756568823d1d490c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Official Form Register" sheetId="2" r:id="R6e47116ab69e4d62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Mapping" sheetId="3" r:id="R6be711c209314461"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COA Document Rules" sheetId="4" r:id="R4e0b0f992e0841ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Practical Tests" sheetId="5" r:id="Rc947c20059534bc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercises and Owners" sheetId="6" r:id="R888dbe7fe3b74fd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Cycles" sheetId="7" r:id="Rcb4325ee6a5e4c59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Rehearsal" sheetId="8" r:id="R482268c8983e4cd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" r:id="Rb623e8eaa4814542"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Summary" sheetId="10" r:id="Rc558a1728dd74274"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Scope" sheetId="11" r:id="R34d850e73da046a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rb85ba7652a3c4d08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Official Form Register" sheetId="2" r:id="R263f11a82a504e34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Mapping" sheetId="3" r:id="R2742b80c1f3a4887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COA Document Rules" sheetId="4" r:id="R81931cbf5cfe44b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Practical Tests" sheetId="5" r:id="R0f384dfc68e1464d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercises and Owners" sheetId="6" r:id="R0ff028ee9f4b4fec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Cycles" sheetId="7" r:id="Rab7656b219d64f0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Rehearsal" sheetId="8" r:id="Ra107c76c16dc4bf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" r:id="Re21de251796a4569"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Summary" sheetId="10" r:id="R836dd742da8f4f2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Scope" sheetId="11" r:id="R268d2a787fef4543"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1270,32 +1270,34 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OfficialFormRegister" displayName="OfficialFormRegister" ref="A5:O36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:O36"/>
-  <x:tableColumns count="15">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OfficialFormRegister" displayName="OfficialFormRegister" ref="A5:Q36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:Q36"/>
+  <x:tableColumns count="17">
     <x:tableColumn id="1" name="Family"/>
     <x:tableColumn id="2" name="Form number"/>
     <x:tableColumn id="3" name="Official title"/>
     <x:tableColumn id="4" name="Manual phase"/>
     <x:tableColumn id="5" name="Sequence"/>
-    <x:tableColumn id="6" name="Starter owner / signatory note"/>
-    <x:tableColumn id="7" name="Process use"/>
-    <x:tableColumn id="8" name="GRAND area"/>
-    <x:tableColumn id="9" name="Applicability status"/>
-    <x:tableColumn id="10" name="Official source"/>
-    <x:tableColumn id="11" name="Local accepted reference"/>
-    <x:tableColumn id="12" name="Current revision / effectivity"/>
-    <x:tableColumn id="13" name="Delivery mode"/>
-    <x:tableColumn id="14" name="Local form owner"/>
-    <x:tableColumn id="15" name="Notes / differences"/>
+    <x:tableColumn id="6" name="Printed manual page(s)"/>
+    <x:tableColumn id="7" name="PDF page(s)"/>
+    <x:tableColumn id="8" name="Starter owner / signatory note"/>
+    <x:tableColumn id="9" name="Process use"/>
+    <x:tableColumn id="10" name="GRAND area"/>
+    <x:tableColumn id="11" name="Applicability status"/>
+    <x:tableColumn id="12" name="Official source"/>
+    <x:tableColumn id="13" name="Local accepted reference"/>
+    <x:tableColumn id="14" name="Current revision / effectivity"/>
+    <x:tableColumn id="15" name="Delivery mode"/>
+    <x:tableColumn id="16" name="Local form owner"/>
+    <x:tableColumn id="17" name="Notes / differences"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FieldMapping" displayName="FieldMapping" ref="A5:O30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:O30"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FieldMapping" displayName="FieldMapping" ref="A5:O75" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:O75"/>
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="Form"/>
     <x:tableColumn id="2" name="Section"/>
@@ -1769,7 +1771,7 @@
         <x:v>Workbook version</x:v>
       </x:c>
       <x:c r="H8" s="158" t="str">
-        <x:v>Starter v1</x:v>
+        <x:v>Starter v1.1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2038,7 +2040,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec0d0c5891244acd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68111b9f1cc243ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2144,7 +2146,7 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C8" s="131" t="n">
-        <x:f>COUNTIF('Official Form Register'!I6:I36,"Accepted - local")</x:f>
+        <x:f>COUNTIF('Official Form Register'!K6:K36,"Accepted - local")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="131" t="n">
@@ -2162,19 +2164,19 @@
         <x:v>Candidate field mappings</x:v>
       </x:c>
       <x:c r="B9" s="132" t="n">
-        <x:f>COUNTA('Field Mapping'!N6:N30)</x:f>
-        <x:v>25</x:v>
+        <x:f>COUNTA('Field Mapping'!N6:N75)</x:f>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C9" s="132" t="n">
-        <x:f>COUNTIF('Field Mapping'!J6:J30,"Accepted - local")</x:f>
+        <x:f>COUNTIF('Field Mapping'!J6:J75,"Accepted - local")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="132" t="n">
         <x:f>B9-C9</x:f>
-        <x:v>25</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E9" s="92" t="str">
-        <x:v>Starter rows cover representative fields; accepted mappings must follow the exact retained local form.</x:v>
+        <x:v>Official-source starter structures cover every listed form; accepted mappings must still follow the exact retained local form.</x:v>
       </x:c>
       <x:c r="F9" s="148"/>
       <x:c r="G9" s="148"/>
@@ -2742,7 +2744,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc319b5ca16fa4b16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R961e16d08b464e77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2756,16 +2758,18 @@
     <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="25" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="25" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="28" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="38" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="22" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -2786,10 +2790,12 @@
       <x:c r="M1" s="146"/>
       <x:c r="N1" s="146"/>
       <x:c r="O1" s="146"/>
+      <x:c r="P1" s="146"/>
+      <x:c r="Q1" s="146"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="147" t="str">
-        <x:v>Starter inventory from the DBM Budget Operations Manual for LGUs, 2023 Edition. Manual-page numbering and current local applicability must be verified against the retained source and local issuances.</x:v>
+        <x:v>Starter inventory from the DBM Budget Operations Manual for LGUs, 2023 Edition. Printed-manual and PDF page anchors were verified against the retained official PDF; current local applicability still requires local confirmation.</x:v>
       </x:c>
       <x:c r="B2" s="147"/>
       <x:c r="C2" s="147"/>
@@ -2805,6 +2811,8 @@
       <x:c r="M2" s="147"/>
       <x:c r="N2" s="147"/>
       <x:c r="O2" s="147"/>
+      <x:c r="P2" s="147"/>
+      <x:c r="Q2" s="147"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="148"/>
@@ -2822,6 +2830,8 @@
       <x:c r="M3" s="148"/>
       <x:c r="N3" s="148"/>
       <x:c r="O3" s="148"/>
+      <x:c r="P3" s="148"/>
+      <x:c r="Q3" s="148"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="148"/>
@@ -2839,6 +2849,8 @@
       <x:c r="M4" s="148"/>
       <x:c r="N4" s="148"/>
       <x:c r="O4" s="148"/>
+      <x:c r="P4" s="148"/>
+      <x:c r="Q4" s="148"/>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
       <x:c r="A5" s="160" t="str">
@@ -2857,33 +2869,39 @@
         <x:v>Sequence</x:v>
       </x:c>
       <x:c r="F5" s="161" t="str">
+        <x:v>Printed manual page(s)</x:v>
+      </x:c>
+      <x:c r="G5" s="161" t="str">
+        <x:v>PDF page(s)</x:v>
+      </x:c>
+      <x:c r="H5" s="161" t="str">
         <x:v>Starter owner / signatory note</x:v>
       </x:c>
-      <x:c r="G5" s="161" t="str">
+      <x:c r="I5" s="161" t="str">
         <x:v>Process use</x:v>
       </x:c>
-      <x:c r="H5" s="161" t="str">
+      <x:c r="J5" s="161" t="str">
         <x:v>GRAND area</x:v>
       </x:c>
-      <x:c r="I5" s="161" t="str">
+      <x:c r="K5" s="161" t="str">
         <x:v>Applicability status</x:v>
       </x:c>
-      <x:c r="J5" s="161" t="str">
+      <x:c r="L5" s="161" t="str">
         <x:v>Official source</x:v>
       </x:c>
-      <x:c r="K5" s="161" t="str">
+      <x:c r="M5" s="161" t="str">
         <x:v>Local accepted reference</x:v>
       </x:c>
-      <x:c r="L5" s="161" t="str">
+      <x:c r="N5" s="161" t="str">
         <x:v>Current revision / effectivity</x:v>
       </x:c>
-      <x:c r="M5" s="161" t="str">
+      <x:c r="O5" s="161" t="str">
         <x:v>Delivery mode</x:v>
       </x:c>
-      <x:c r="N5" s="161" t="str">
+      <x:c r="P5" s="161" t="str">
         <x:v>Local form owner</x:v>
       </x:c>
-      <x:c r="O5" s="162" t="str">
+      <x:c r="Q5" s="162" t="str">
         <x:v>Notes / differences</x:v>
       </x:c>
     </x:row>
@@ -2904,25 +2922,31 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F6" s="56" t="str">
+        <x:v>59–61</x:v>
+      </x:c>
+      <x:c r="G6" s="56" t="str">
+        <x:v>74–76</x:v>
+      </x:c>
+      <x:c r="H6" s="56" t="str">
         <x:v>Local Finance Committee and Local Accountant; approved by LCE</x:v>
       </x:c>
-      <x:c r="G6" s="56" t="str">
+      <x:c r="I6" s="56" t="str">
         <x:v>Annual budget preparation</x:v>
       </x:c>
-      <x:c r="H6" s="56" t="str">
+      <x:c r="J6" s="56" t="str">
         <x:v>F3 annual budget / F9 reporting</x:v>
       </x:c>
-      <x:c r="I6" s="62" t="str">
+      <x:c r="K6" s="62" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J6" s="56" t="str">
+      <x:c r="L6" s="56" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K6" s="62" t="str"/>
-      <x:c r="L6" s="62" t="str"/>
       <x:c r="M6" s="62" t="str"/>
       <x:c r="N6" s="62" t="str"/>
       <x:c r="O6" s="62" t="str"/>
+      <x:c r="P6" s="62" t="str"/>
+      <x:c r="Q6" s="62" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="57" t="str">
@@ -2941,25 +2965,31 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="F7" s="57" t="str">
+        <x:v>62–63</x:v>
+      </x:c>
+      <x:c r="G7" s="57" t="str">
+        <x:v>77–78</x:v>
+      </x:c>
+      <x:c r="H7" s="57" t="str">
         <x:v>Department Head; reviewed by LBO; approved by LCE</x:v>
       </x:c>
-      <x:c r="G7" s="57" t="str">
+      <x:c r="I7" s="57" t="str">
         <x:v>Department proposal</x:v>
       </x:c>
-      <x:c r="H7" s="57" t="str">
+      <x:c r="J7" s="57" t="str">
         <x:v>F3 annual budget</x:v>
       </x:c>
-      <x:c r="I7" s="63" t="str">
+      <x:c r="K7" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J7" s="57" t="str">
+      <x:c r="L7" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K7" s="63" t="str"/>
-      <x:c r="L7" s="63" t="str"/>
       <x:c r="M7" s="63" t="str"/>
       <x:c r="N7" s="63" t="str"/>
       <x:c r="O7" s="63" t="str"/>
+      <x:c r="P7" s="63" t="str"/>
+      <x:c r="Q7" s="63" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="57" t="str">
@@ -2978,25 +3008,31 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F8" s="57" t="str">
+        <x:v>64–66</x:v>
+      </x:c>
+      <x:c r="G8" s="57" t="str">
+        <x:v>79–81</x:v>
+      </x:c>
+      <x:c r="H8" s="57" t="str">
         <x:v>HRMO; reviewed by LBO; approved by LCE</x:v>
       </x:c>
-      <x:c r="G8" s="57" t="str">
+      <x:c r="I8" s="57" t="str">
         <x:v>Personnel proposal</x:v>
       </x:c>
-      <x:c r="H8" s="57" t="str">
+      <x:c r="J8" s="57" t="str">
         <x:v>F3 annual budget</x:v>
       </x:c>
-      <x:c r="I8" s="63" t="str">
+      <x:c r="K8" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J8" s="57" t="str">
+      <x:c r="L8" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K8" s="63" t="str"/>
-      <x:c r="L8" s="63" t="str"/>
       <x:c r="M8" s="63" t="str"/>
       <x:c r="N8" s="63" t="str"/>
       <x:c r="O8" s="63" t="str"/>
+      <x:c r="P8" s="63" t="str"/>
+      <x:c r="Q8" s="63" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="57" t="str">
@@ -3015,25 +3051,31 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F9" s="57" t="str">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="G9" s="57" t="str">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="H9" s="57" t="str">
         <x:v>Department Head; reviewed by LFC; approved by LCE</x:v>
       </x:c>
-      <x:c r="G9" s="57" t="str">
+      <x:c r="I9" s="57" t="str">
         <x:v>Performance-informed proposal</x:v>
       </x:c>
-      <x:c r="H9" s="57" t="str">
+      <x:c r="J9" s="57" t="str">
         <x:v>F3 annual budget</x:v>
       </x:c>
-      <x:c r="I9" s="63" t="str">
+      <x:c r="K9" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J9" s="57" t="str">
+      <x:c r="L9" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K9" s="63" t="str"/>
-      <x:c r="L9" s="63" t="str"/>
       <x:c r="M9" s="63" t="str"/>
       <x:c r="N9" s="63" t="str"/>
       <x:c r="O9" s="63" t="str"/>
+      <x:c r="P9" s="63" t="str"/>
+      <x:c r="Q9" s="63" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="57" t="str">
@@ -3052,25 +3094,31 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="F10" s="57" t="str">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="G10" s="57" t="str">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="H10" s="57" t="str">
         <x:v>Local Accountant; noted by LCE</x:v>
       </x:c>
-      <x:c r="G10" s="57" t="str">
+      <x:c r="I10" s="57" t="str">
         <x:v>Debt disclosure</x:v>
       </x:c>
-      <x:c r="H10" s="57" t="str">
+      <x:c r="J10" s="57" t="str">
         <x:v>F3/F9</x:v>
       </x:c>
-      <x:c r="I10" s="63" t="str">
+      <x:c r="K10" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J10" s="57" t="str">
+      <x:c r="L10" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K10" s="63" t="str"/>
-      <x:c r="L10" s="63" t="str"/>
       <x:c r="M10" s="63" t="str"/>
       <x:c r="N10" s="63" t="str"/>
       <x:c r="O10" s="63" t="str"/>
+      <x:c r="P10" s="63" t="str"/>
+      <x:c r="Q10" s="63" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="57" t="str">
@@ -3089,25 +3137,31 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="F11" s="57" t="str">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="G11" s="57" t="str">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="H11" s="57" t="str">
         <x:v>Local Finance Committee; approved by LCE</x:v>
       </x:c>
-      <x:c r="G11" s="57" t="str">
+      <x:c r="I11" s="57" t="str">
         <x:v>Mandatory requirements</x:v>
       </x:c>
-      <x:c r="H11" s="57" t="str">
+      <x:c r="J11" s="57" t="str">
         <x:v>F3 annual budget</x:v>
       </x:c>
-      <x:c r="I11" s="63" t="str">
+      <x:c r="K11" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J11" s="57" t="str">
+      <x:c r="L11" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K11" s="63" t="str"/>
-      <x:c r="L11" s="63" t="str"/>
       <x:c r="M11" s="63" t="str"/>
       <x:c r="N11" s="63" t="str"/>
       <x:c r="O11" s="63" t="str"/>
+      <x:c r="P11" s="63" t="str"/>
+      <x:c r="Q11" s="63" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="57" t="str">
@@ -3126,25 +3180,31 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="F12" s="57" t="str">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="G12" s="57" t="str">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="H12" s="57" t="str">
         <x:v>Local Budget Officer; approved by LCE</x:v>
       </x:c>
-      <x:c r="G12" s="57" t="str">
+      <x:c r="I12" s="57" t="str">
         <x:v>Sector allocation</x:v>
       </x:c>
-      <x:c r="H12" s="57" t="str">
+      <x:c r="J12" s="57" t="str">
         <x:v>F3/F9</x:v>
       </x:c>
-      <x:c r="I12" s="63" t="str">
+      <x:c r="K12" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J12" s="57" t="str">
+      <x:c r="L12" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K12" s="63" t="str"/>
-      <x:c r="L12" s="63" t="str"/>
       <x:c r="M12" s="63" t="str"/>
       <x:c r="N12" s="63" t="str"/>
       <x:c r="O12" s="63" t="str"/>
+      <x:c r="P12" s="63" t="str"/>
+      <x:c r="Q12" s="63" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="57" t="str">
@@ -3163,25 +3223,31 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="F13" s="57" t="str">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="G13" s="57" t="str">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="H13" s="57" t="str">
         <x:v>Local Treasurer and/or Local Accountant, depending on source</x:v>
       </x:c>
-      <x:c r="G13" s="57" t="str">
+      <x:c r="I13" s="57" t="str">
         <x:v>Supplemental funding</x:v>
       </x:c>
-      <x:c r="H13" s="57" t="str">
+      <x:c r="J13" s="57" t="str">
         <x:v>F3 budget adjustment</x:v>
       </x:c>
-      <x:c r="I13" s="63" t="str">
+      <x:c r="K13" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J13" s="57" t="str">
+      <x:c r="L13" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K13" s="63" t="str"/>
-      <x:c r="L13" s="63" t="str"/>
       <x:c r="M13" s="63" t="str"/>
       <x:c r="N13" s="63" t="str"/>
       <x:c r="O13" s="63" t="str"/>
+      <x:c r="P13" s="63" t="str"/>
+      <x:c r="Q13" s="63" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="57" t="str">
@@ -3200,25 +3266,31 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="F14" s="57" t="str">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="G14" s="57" t="str">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="H14" s="57" t="str">
         <x:v>Local Budget Officer; approved by LCE</x:v>
       </x:c>
-      <x:c r="G14" s="57" t="str">
+      <x:c r="I14" s="57" t="str">
         <x:v>Supplemental appropriation</x:v>
       </x:c>
-      <x:c r="H14" s="57" t="str">
+      <x:c r="J14" s="57" t="str">
         <x:v>F3 budget adjustment</x:v>
       </x:c>
-      <x:c r="I14" s="63" t="str">
+      <x:c r="K14" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J14" s="57" t="str">
+      <x:c r="L14" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K14" s="63" t="str"/>
-      <x:c r="L14" s="63" t="str"/>
       <x:c r="M14" s="63" t="str"/>
       <x:c r="N14" s="63" t="str"/>
       <x:c r="O14" s="63" t="str"/>
+      <x:c r="P14" s="63" t="str"/>
+      <x:c r="Q14" s="63" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="57" t="str">
@@ -3237,25 +3309,31 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F15" s="57" t="str">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="G15" s="57" t="str">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="H15" s="57" t="str">
         <x:v>Confirm from current manual and local route</x:v>
       </x:c>
-      <x:c r="G15" s="57" t="str">
+      <x:c r="I15" s="57" t="str">
         <x:v>Annual budget enactment</x:v>
       </x:c>
-      <x:c r="H15" s="57" t="str">
+      <x:c r="J15" s="57" t="str">
         <x:v>F3/F10</x:v>
       </x:c>
-      <x:c r="I15" s="63" t="str">
+      <x:c r="K15" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J15" s="57" t="str">
+      <x:c r="L15" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K15" s="63" t="str"/>
-      <x:c r="L15" s="63" t="str"/>
       <x:c r="M15" s="63" t="str"/>
       <x:c r="N15" s="63" t="str"/>
       <x:c r="O15" s="63" t="str"/>
+      <x:c r="P15" s="63" t="str"/>
+      <x:c r="Q15" s="63" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="57" t="str">
@@ -3274,25 +3352,31 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="F16" s="57" t="str">
+        <x:v>110–111</x:v>
+      </x:c>
+      <x:c r="G16" s="57" t="str">
+        <x:v>125–126</x:v>
+      </x:c>
+      <x:c r="H16" s="57" t="str">
         <x:v>Confirm from current manual and local route</x:v>
       </x:c>
-      <x:c r="G16" s="57" t="str">
+      <x:c r="I16" s="57" t="str">
         <x:v>Supplemental budget enactment</x:v>
       </x:c>
-      <x:c r="H16" s="57" t="str">
+      <x:c r="J16" s="57" t="str">
         <x:v>F3/F10</x:v>
       </x:c>
-      <x:c r="I16" s="63" t="str">
+      <x:c r="K16" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J16" s="57" t="str">
+      <x:c r="L16" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K16" s="63" t="str"/>
-      <x:c r="L16" s="63" t="str"/>
       <x:c r="M16" s="63" t="str"/>
       <x:c r="N16" s="63" t="str"/>
       <x:c r="O16" s="63" t="str"/>
+      <x:c r="P16" s="63" t="str"/>
+      <x:c r="Q16" s="63" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="57" t="str">
@@ -3311,25 +3395,31 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="F17" s="57" t="str">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="G17" s="57" t="str">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="H17" s="57" t="str">
         <x:v>Reviewing authority; confirm current route</x:v>
       </x:c>
-      <x:c r="G17" s="57" t="str">
+      <x:c r="I17" s="57" t="str">
         <x:v>Annual budget review</x:v>
       </x:c>
-      <x:c r="H17" s="57" t="str">
+      <x:c r="J17" s="57" t="str">
         <x:v>F3/F10</x:v>
       </x:c>
-      <x:c r="I17" s="63" t="str">
+      <x:c r="K17" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J17" s="57" t="str">
+      <x:c r="L17" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K17" s="63" t="str"/>
-      <x:c r="L17" s="63" t="str"/>
       <x:c r="M17" s="63" t="str"/>
       <x:c r="N17" s="63" t="str"/>
       <x:c r="O17" s="63" t="str"/>
+      <x:c r="P17" s="63" t="str"/>
+      <x:c r="Q17" s="63" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="57" t="str">
@@ -3348,25 +3438,31 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="F18" s="57" t="str">
+        <x:v>137–138</x:v>
+      </x:c>
+      <x:c r="G18" s="57" t="str">
+        <x:v>152–153</x:v>
+      </x:c>
+      <x:c r="H18" s="57" t="str">
         <x:v>Reviewing authority; confirm current route</x:v>
       </x:c>
-      <x:c r="G18" s="57" t="str">
+      <x:c r="I18" s="57" t="str">
         <x:v>Supplemental budget review</x:v>
       </x:c>
-      <x:c r="H18" s="57" t="str">
+      <x:c r="J18" s="57" t="str">
         <x:v>F3/F10</x:v>
       </x:c>
-      <x:c r="I18" s="63" t="str">
+      <x:c r="K18" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J18" s="57" t="str">
+      <x:c r="L18" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K18" s="63" t="str"/>
-      <x:c r="L18" s="63" t="str"/>
       <x:c r="M18" s="63" t="str"/>
       <x:c r="N18" s="63" t="str"/>
       <x:c r="O18" s="63" t="str"/>
+      <x:c r="P18" s="63" t="str"/>
+      <x:c r="Q18" s="63" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="57" t="str">
@@ -3385,25 +3481,31 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="F19" s="57" t="str">
+        <x:v>139–152</x:v>
+      </x:c>
+      <x:c r="G19" s="57" t="str">
+        <x:v>154–167</x:v>
+      </x:c>
+      <x:c r="H19" s="57" t="str">
         <x:v>Reviewing authority; confirm current route</x:v>
       </x:c>
-      <x:c r="G19" s="57" t="str">
+      <x:c r="I19" s="57" t="str">
         <x:v>Review findings</x:v>
       </x:c>
-      <x:c r="H19" s="57" t="str">
+      <x:c r="J19" s="57" t="str">
         <x:v>F3/F10</x:v>
       </x:c>
-      <x:c r="I19" s="63" t="str">
+      <x:c r="K19" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J19" s="57" t="str">
+      <x:c r="L19" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K19" s="63" t="str"/>
-      <x:c r="L19" s="63" t="str"/>
       <x:c r="M19" s="63" t="str"/>
       <x:c r="N19" s="63" t="str"/>
       <x:c r="O19" s="63" t="str"/>
+      <x:c r="P19" s="63" t="str"/>
+      <x:c r="Q19" s="63" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="57" t="str">
@@ -3422,25 +3524,31 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F20" s="57" t="str">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="G20" s="57" t="str">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="H20" s="57" t="str">
         <x:v>Reviewing authority; confirm current route</x:v>
       </x:c>
-      <x:c r="G20" s="57" t="str">
+      <x:c r="I20" s="57" t="str">
         <x:v>PS review</x:v>
       </x:c>
-      <x:c r="H20" s="57" t="str">
+      <x:c r="J20" s="57" t="str">
         <x:v>F3/F10</x:v>
       </x:c>
-      <x:c r="I20" s="63" t="str">
+      <x:c r="K20" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J20" s="57" t="str">
+      <x:c r="L20" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K20" s="63" t="str"/>
-      <x:c r="L20" s="63" t="str"/>
       <x:c r="M20" s="63" t="str"/>
       <x:c r="N20" s="63" t="str"/>
       <x:c r="O20" s="63" t="str"/>
+      <x:c r="P20" s="63" t="str"/>
+      <x:c r="Q20" s="63" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="57" t="str">
@@ -3459,25 +3567,31 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="F21" s="57" t="str">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="G21" s="57" t="str">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="H21" s="57" t="str">
         <x:v>Reviewing authority; confirm current route</x:v>
       </x:c>
-      <x:c r="G21" s="57" t="str">
+      <x:c r="I21" s="57" t="str">
         <x:v>PS limitation review</x:v>
       </x:c>
-      <x:c r="H21" s="57" t="str">
+      <x:c r="J21" s="57" t="str">
         <x:v>F3/F10</x:v>
       </x:c>
-      <x:c r="I21" s="63" t="str">
+      <x:c r="K21" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J21" s="57" t="str">
+      <x:c r="L21" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K21" s="63" t="str"/>
-      <x:c r="L21" s="63" t="str"/>
       <x:c r="M21" s="63" t="str"/>
       <x:c r="N21" s="63" t="str"/>
       <x:c r="O21" s="63" t="str"/>
+      <x:c r="P21" s="63" t="str"/>
+      <x:c r="Q21" s="63" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="57" t="str">
@@ -3496,25 +3610,31 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="F22" s="57" t="str">
+        <x:v>178–179</x:v>
+      </x:c>
+      <x:c r="G22" s="57" t="str">
+        <x:v>193–194</x:v>
+      </x:c>
+      <x:c r="H22" s="57" t="str">
         <x:v>LBO recommendation; LCE approval</x:v>
       </x:c>
-      <x:c r="G22" s="57" t="str">
+      <x:c r="I22" s="57" t="str">
         <x:v>Allotment release</x:v>
       </x:c>
-      <x:c r="H22" s="57" t="str">
+      <x:c r="J22" s="57" t="str">
         <x:v>F4 allotment control</x:v>
       </x:c>
-      <x:c r="I22" s="63" t="str">
+      <x:c r="K22" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J22" s="57" t="str">
+      <x:c r="L22" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K22" s="63" t="str"/>
-      <x:c r="L22" s="63" t="str"/>
       <x:c r="M22" s="63" t="str"/>
       <x:c r="N22" s="63" t="str"/>
       <x:c r="O22" s="63" t="str"/>
+      <x:c r="P22" s="63" t="str"/>
+      <x:c r="Q22" s="63" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="57" t="str">
@@ -3533,25 +3653,31 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="F23" s="57" t="str">
+        <x:v>180–181</x:v>
+      </x:c>
+      <x:c r="G23" s="57" t="str">
+        <x:v>195–196</x:v>
+      </x:c>
+      <x:c r="H23" s="57" t="str">
         <x:v>LBO recommendation; LCE approval</x:v>
       </x:c>
-      <x:c r="G23" s="57" t="str">
+      <x:c r="I23" s="57" t="str">
         <x:v>Allotment release</x:v>
       </x:c>
-      <x:c r="H23" s="57" t="str">
+      <x:c r="J23" s="57" t="str">
         <x:v>F4 allotment control</x:v>
       </x:c>
-      <x:c r="I23" s="63" t="str">
+      <x:c r="K23" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J23" s="57" t="str">
+      <x:c r="L23" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K23" s="63" t="str"/>
-      <x:c r="L23" s="63" t="str"/>
       <x:c r="M23" s="63" t="str"/>
       <x:c r="N23" s="63" t="str"/>
       <x:c r="O23" s="63" t="str"/>
+      <x:c r="P23" s="63" t="str"/>
+      <x:c r="Q23" s="63" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="57" t="str">
@@ -3570,25 +3696,31 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="F24" s="57" t="str">
+        <x:v>182–183</x:v>
+      </x:c>
+      <x:c r="G24" s="57" t="str">
+        <x:v>197–198</x:v>
+      </x:c>
+      <x:c r="H24" s="57" t="str">
         <x:v>LBO recommendation; LCE approval</x:v>
       </x:c>
-      <x:c r="G24" s="57" t="str">
+      <x:c r="I24" s="57" t="str">
         <x:v>Allotment release</x:v>
       </x:c>
-      <x:c r="H24" s="57" t="str">
+      <x:c r="J24" s="57" t="str">
         <x:v>F4 allotment control</x:v>
       </x:c>
-      <x:c r="I24" s="63" t="str">
+      <x:c r="K24" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J24" s="57" t="str">
+      <x:c r="L24" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K24" s="63" t="str"/>
-      <x:c r="L24" s="63" t="str"/>
       <x:c r="M24" s="63" t="str"/>
       <x:c r="N24" s="63" t="str"/>
       <x:c r="O24" s="63" t="str"/>
+      <x:c r="P24" s="63" t="str"/>
+      <x:c r="Q24" s="63" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="57" t="str">
@@ -3607,25 +3739,31 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="F25" s="57" t="str">
+        <x:v>184–185</x:v>
+      </x:c>
+      <x:c r="G25" s="57" t="str">
+        <x:v>199–200</x:v>
+      </x:c>
+      <x:c r="H25" s="57" t="str">
         <x:v>LBO recommendation; LCE approval</x:v>
       </x:c>
-      <x:c r="G25" s="57" t="str">
+      <x:c r="I25" s="57" t="str">
         <x:v>Allotment release</x:v>
       </x:c>
-      <x:c r="H25" s="57" t="str">
+      <x:c r="J25" s="57" t="str">
         <x:v>F4 allotment control</x:v>
       </x:c>
-      <x:c r="I25" s="63" t="str">
+      <x:c r="K25" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J25" s="57" t="str">
+      <x:c r="L25" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K25" s="63" t="str"/>
-      <x:c r="L25" s="63" t="str"/>
       <x:c r="M25" s="63" t="str"/>
       <x:c r="N25" s="63" t="str"/>
       <x:c r="O25" s="63" t="str"/>
+      <x:c r="P25" s="63" t="str"/>
+      <x:c r="Q25" s="63" t="str"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="57" t="str">
@@ -3644,25 +3782,31 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="F26" s="57" t="str">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="G26" s="57" t="str">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="H26" s="57" t="str">
         <x:v>Confirm authority, savings source, use, and local approval route</x:v>
       </x:c>
-      <x:c r="G26" s="57" t="str">
+      <x:c r="I26" s="57" t="str">
         <x:v>Augmentation</x:v>
       </x:c>
-      <x:c r="H26" s="57" t="str">
+      <x:c r="J26" s="57" t="str">
         <x:v>F4 adjustment control</x:v>
       </x:c>
-      <x:c r="I26" s="63" t="str">
+      <x:c r="K26" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J26" s="57" t="str">
+      <x:c r="L26" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K26" s="63" t="str"/>
-      <x:c r="L26" s="63" t="str"/>
       <x:c r="M26" s="63" t="str"/>
       <x:c r="N26" s="63" t="str"/>
       <x:c r="O26" s="63" t="str"/>
+      <x:c r="P26" s="63" t="str"/>
+      <x:c r="Q26" s="63" t="str"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="57" t="str">
@@ -3681,25 +3825,31 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="F27" s="57" t="str">
+        <x:v>187–188</x:v>
+      </x:c>
+      <x:c r="G27" s="57" t="str">
+        <x:v>202–203</x:v>
+      </x:c>
+      <x:c r="H27" s="57" t="str">
         <x:v>Confirm from current manual and local route</x:v>
       </x:c>
-      <x:c r="G27" s="57" t="str">
+      <x:c r="I27" s="57" t="str">
         <x:v>Reenacted budget</x:v>
       </x:c>
-      <x:c r="H27" s="57" t="str">
+      <x:c r="J27" s="57" t="str">
         <x:v>F3/F4</x:v>
       </x:c>
-      <x:c r="I27" s="63" t="str">
+      <x:c r="K27" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J27" s="57" t="str">
+      <x:c r="L27" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K27" s="63" t="str"/>
-      <x:c r="L27" s="63" t="str"/>
       <x:c r="M27" s="63" t="str"/>
       <x:c r="N27" s="63" t="str"/>
       <x:c r="O27" s="63" t="str"/>
+      <x:c r="P27" s="63" t="str"/>
+      <x:c r="Q27" s="63" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="57" t="str">
@@ -3718,25 +3868,31 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="F28" s="57" t="str">
+        <x:v>189–190</x:v>
+      </x:c>
+      <x:c r="G28" s="57" t="str">
+        <x:v>204–205</x:v>
+      </x:c>
+      <x:c r="H28" s="57" t="str">
         <x:v>Confirm from current manual and local route</x:v>
       </x:c>
-      <x:c r="G28" s="57" t="str">
+      <x:c r="I28" s="57" t="str">
         <x:v>Reenacted budget</x:v>
       </x:c>
-      <x:c r="H28" s="57" t="str">
+      <x:c r="J28" s="57" t="str">
         <x:v>F3/F4</x:v>
       </x:c>
-      <x:c r="I28" s="63" t="str">
+      <x:c r="K28" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J28" s="57" t="str">
+      <x:c r="L28" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K28" s="63" t="str"/>
-      <x:c r="L28" s="63" t="str"/>
       <x:c r="M28" s="63" t="str"/>
       <x:c r="N28" s="63" t="str"/>
       <x:c r="O28" s="63" t="str"/>
+      <x:c r="P28" s="63" t="str"/>
+      <x:c r="Q28" s="63" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="57" t="str">
@@ -3755,25 +3911,31 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="F29" s="57" t="str">
+        <x:v>191–192</x:v>
+      </x:c>
+      <x:c r="G29" s="57" t="str">
+        <x:v>206–207</x:v>
+      </x:c>
+      <x:c r="H29" s="57" t="str">
         <x:v>Confirm from current manual and local route</x:v>
       </x:c>
-      <x:c r="G29" s="57" t="str">
+      <x:c r="I29" s="57" t="str">
         <x:v>Performance targets</x:v>
       </x:c>
-      <x:c r="H29" s="57" t="str">
+      <x:c r="J29" s="57" t="str">
         <x:v>F3/F9</x:v>
       </x:c>
-      <x:c r="I29" s="63" t="str">
+      <x:c r="K29" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J29" s="57" t="str">
+      <x:c r="L29" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K29" s="63" t="str"/>
-      <x:c r="L29" s="63" t="str"/>
       <x:c r="M29" s="63" t="str"/>
       <x:c r="N29" s="63" t="str"/>
       <x:c r="O29" s="63" t="str"/>
+      <x:c r="P29" s="63" t="str"/>
+      <x:c r="Q29" s="63" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="57" t="str">
@@ -3792,25 +3954,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="F30" s="57" t="str">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="G30" s="57" t="str">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="H30" s="57" t="str">
         <x:v>Confirm from current manual and local route</x:v>
       </x:c>
-      <x:c r="G30" s="57" t="str">
+      <x:c r="I30" s="57" t="str">
         <x:v>Detailed targets</x:v>
       </x:c>
-      <x:c r="H30" s="57" t="str">
+      <x:c r="J30" s="57" t="str">
         <x:v>F3/F9</x:v>
       </x:c>
-      <x:c r="I30" s="63" t="str">
+      <x:c r="K30" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J30" s="57" t="str">
+      <x:c r="L30" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K30" s="63" t="str"/>
-      <x:c r="L30" s="63" t="str"/>
       <x:c r="M30" s="63" t="str"/>
       <x:c r="N30" s="63" t="str"/>
       <x:c r="O30" s="63" t="str"/>
+      <x:c r="P30" s="63" t="str"/>
+      <x:c r="Q30" s="63" t="str"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="57" t="str">
@@ -3829,25 +3997,31 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="F31" s="57" t="str">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="G31" s="57" t="str">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="H31" s="57" t="str">
         <x:v>Local Treasurer prepares; Local Accountant certifies</x:v>
       </x:c>
-      <x:c r="G31" s="57" t="str">
+      <x:c r="I31" s="57" t="str">
         <x:v>Quarterly receipts</x:v>
       </x:c>
-      <x:c r="H31" s="57" t="str">
+      <x:c r="J31" s="57" t="str">
         <x:v>F9 accountability reports</x:v>
       </x:c>
-      <x:c r="I31" s="63" t="str">
+      <x:c r="K31" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J31" s="57" t="str">
+      <x:c r="L31" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K31" s="63" t="str"/>
-      <x:c r="L31" s="63" t="str"/>
       <x:c r="M31" s="63" t="str"/>
       <x:c r="N31" s="63" t="str"/>
       <x:c r="O31" s="63" t="str"/>
+      <x:c r="P31" s="63" t="str"/>
+      <x:c r="Q31" s="63" t="str"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="57" t="str">
@@ -3866,25 +4040,31 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="F32" s="57" t="str">
+        <x:v>206–207</x:v>
+      </x:c>
+      <x:c r="G32" s="57" t="str">
+        <x:v>221–222</x:v>
+      </x:c>
+      <x:c r="H32" s="57" t="str">
         <x:v>Confirm from current manual and local route</x:v>
       </x:c>
-      <x:c r="G32" s="57" t="str">
+      <x:c r="I32" s="57" t="str">
         <x:v>Quarterly financial operations</x:v>
       </x:c>
-      <x:c r="H32" s="57" t="str">
+      <x:c r="J32" s="57" t="str">
         <x:v>F9 accountability reports</x:v>
       </x:c>
-      <x:c r="I32" s="63" t="str">
+      <x:c r="K32" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J32" s="57" t="str">
+      <x:c r="L32" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K32" s="63" t="str"/>
-      <x:c r="L32" s="63" t="str"/>
       <x:c r="M32" s="63" t="str"/>
       <x:c r="N32" s="63" t="str"/>
       <x:c r="O32" s="63" t="str"/>
+      <x:c r="P32" s="63" t="str"/>
+      <x:c r="Q32" s="63" t="str"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="57" t="str">
@@ -3903,25 +4083,31 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="F33" s="57" t="str">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="G33" s="57" t="str">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="H33" s="57" t="str">
         <x:v>Confirm from current manual and local route</x:v>
       </x:c>
-      <x:c r="G33" s="57" t="str">
+      <x:c r="I33" s="57" t="str">
         <x:v>Quarterly physical operations</x:v>
       </x:c>
-      <x:c r="H33" s="57" t="str">
+      <x:c r="J33" s="57" t="str">
         <x:v>F9 accountability reports</x:v>
       </x:c>
-      <x:c r="I33" s="63" t="str">
+      <x:c r="K33" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J33" s="57" t="str">
+      <x:c r="L33" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K33" s="63" t="str"/>
-      <x:c r="L33" s="63" t="str"/>
       <x:c r="M33" s="63" t="str"/>
       <x:c r="N33" s="63" t="str"/>
       <x:c r="O33" s="63" t="str"/>
+      <x:c r="P33" s="63" t="str"/>
+      <x:c r="Q33" s="63" t="str"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="57" t="str">
@@ -3940,25 +4126,31 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="F34" s="57" t="str">
+        <x:v>209–210</x:v>
+      </x:c>
+      <x:c r="G34" s="57" t="str">
+        <x:v>224–225</x:v>
+      </x:c>
+      <x:c r="H34" s="57" t="str">
         <x:v>Local Treasurer and LBO prepare; Local Accountant certifies; LCE approves</x:v>
       </x:c>
-      <x:c r="G34" s="57" t="str">
+      <x:c r="I34" s="57" t="str">
         <x:v>Annual receipts/expenditures</x:v>
       </x:c>
-      <x:c r="H34" s="57" t="str">
+      <x:c r="J34" s="57" t="str">
         <x:v>F9 accountability reports</x:v>
       </x:c>
-      <x:c r="I34" s="63" t="str">
+      <x:c r="K34" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J34" s="57" t="str">
+      <x:c r="L34" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K34" s="63" t="str"/>
-      <x:c r="L34" s="63" t="str"/>
       <x:c r="M34" s="63" t="str"/>
       <x:c r="N34" s="63" t="str"/>
       <x:c r="O34" s="63" t="str"/>
+      <x:c r="P34" s="63" t="str"/>
+      <x:c r="Q34" s="63" t="str"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="57" t="str">
@@ -3977,25 +4169,31 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="F35" s="57" t="str">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="G35" s="57" t="str">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="H35" s="57" t="str">
         <x:v>Confirm from current manual and local route</x:v>
       </x:c>
-      <x:c r="G35" s="57" t="str">
+      <x:c r="I35" s="57" t="str">
         <x:v>Performance evaluation</x:v>
       </x:c>
-      <x:c r="H35" s="57" t="str">
+      <x:c r="J35" s="57" t="str">
         <x:v>F9 accountability reports</x:v>
       </x:c>
-      <x:c r="I35" s="63" t="str">
+      <x:c r="K35" s="63" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J35" s="57" t="str">
+      <x:c r="L35" s="57" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K35" s="63" t="str"/>
-      <x:c r="L35" s="63" t="str"/>
       <x:c r="M35" s="63" t="str"/>
       <x:c r="N35" s="63" t="str"/>
       <x:c r="O35" s="63" t="str"/>
+      <x:c r="P35" s="63" t="str"/>
+      <x:c r="Q35" s="63" t="str"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="58" t="str">
@@ -4014,32 +4212,38 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="F36" s="58" t="str">
+        <x:v>212–213</x:v>
+      </x:c>
+      <x:c r="G36" s="58" t="str">
+        <x:v>227–228</x:v>
+      </x:c>
+      <x:c r="H36" s="58" t="str">
         <x:v>Confirm from current manual and local route</x:v>
       </x:c>
-      <x:c r="G36" s="58" t="str">
+      <x:c r="I36" s="58" t="str">
         <x:v>Accomplishment monitoring</x:v>
       </x:c>
-      <x:c r="H36" s="58" t="str">
+      <x:c r="J36" s="58" t="str">
         <x:v>F9 accountability reports</x:v>
       </x:c>
-      <x:c r="I36" s="64" t="str">
+      <x:c r="K36" s="64" t="str">
         <x:v>Candidate - confirm locally</x:v>
       </x:c>
-      <x:c r="J36" s="58" t="str">
+      <x:c r="L36" s="58" t="str">
         <x:v>DBM BOM for LGUs, 2023</x:v>
       </x:c>
-      <x:c r="K36" s="64" t="str"/>
-      <x:c r="L36" s="64" t="str"/>
       <x:c r="M36" s="64" t="str"/>
       <x:c r="N36" s="64" t="str"/>
       <x:c r="O36" s="64" t="str"/>
+      <x:c r="P36" s="64" t="str"/>
+      <x:c r="Q36" s="64" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:O1"/>
-    <x:mergeCell ref="A2:O2"/>
+    <x:mergeCell ref="A1:Q1"/>
+    <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="I6:I36">
+  <x:conditionalFormatting sqref="K6:K36">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Accepted"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Pass"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Ready"/>
@@ -4047,16 +4251,16 @@
     <x:cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Fail"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="I6:I36">
+    <x:dataValidation type="list" sqref="K6:K36">
       <x:formula1>"Candidate - confirm locally,Applicable - mapping,Practical testing,Accepted - local,Not applicable - documented"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="M6:M36">
+    <x:dataValidation type="list" sqref="O6:O36">
       <x:formula1>"Print,Download,Both,Data-only / no local form,Confirm locally"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4fca8033cc64deb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cacdf1edeaa40d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4103,7 +4307,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="147" t="str">
-        <x:v>Representative rows are starters, not executable template rules. Add, edit, or remove rows only through the locally governed form-intake process, then retain the accepted mapping version in GRAND.</x:v>
+        <x:v>Official-source starter structures now cover every listed DBM form. They remain non-executable candidates: compare each row with the retained current local form, revise through the governed intake process, and accept only the exact tested mapping in GRAND.</x:v>
       </x:c>
       <x:c r="B2" s="147"/>
       <x:c r="C2" s="147"/>
@@ -4238,7 +4442,9 @@
       <x:c r="N6" s="56" t="str">
         <x:v>MAP-001</x:v>
       </x:c>
-      <x:c r="O6" s="62" t="str"/>
+      <x:c r="O6" s="62" t="str">
+        <x:v>DBM manual pp. 89 (PDF pp. 104)</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="57" t="str">
@@ -4277,7 +4483,9 @@
       <x:c r="N7" s="57" t="str">
         <x:v>MAP-002</x:v>
       </x:c>
-      <x:c r="O7" s="63" t="str"/>
+      <x:c r="O7" s="63" t="str">
+        <x:v>DBM manual pp. 89 (PDF pp. 104)</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="57" t="str">
@@ -4316,7 +4524,9 @@
       <x:c r="N8" s="57" t="str">
         <x:v>MAP-003</x:v>
       </x:c>
-      <x:c r="O8" s="63" t="str"/>
+      <x:c r="O8" s="63" t="str">
+        <x:v>DBM manual pp. 89 (PDF pp. 104)</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="57" t="str">
@@ -4355,7 +4565,9 @@
       <x:c r="N9" s="57" t="str">
         <x:v>MAP-004</x:v>
       </x:c>
-      <x:c r="O9" s="63" t="str"/>
+      <x:c r="O9" s="63" t="str">
+        <x:v>DBM manual pp. 89 (PDF pp. 104)</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="57" t="str">
@@ -4394,7 +4606,9 @@
       <x:c r="N10" s="57" t="str">
         <x:v>MAP-005</x:v>
       </x:c>
-      <x:c r="O10" s="63" t="str"/>
+      <x:c r="O10" s="63" t="str">
+        <x:v>DBM manual pp. 89 (PDF pp. 104)</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="57" t="str">
@@ -4433,7 +4647,9 @@
       <x:c r="N11" s="57" t="str">
         <x:v>MAP-006</x:v>
       </x:c>
-      <x:c r="O11" s="63" t="str"/>
+      <x:c r="O11" s="63" t="str">
+        <x:v>DBM manual pp. 178–179 (PDF pp. 193–194)</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="57" t="str">
@@ -4472,7 +4688,9 @@
       <x:c r="N12" s="57" t="str">
         <x:v>MAP-007</x:v>
       </x:c>
-      <x:c r="O12" s="63" t="str"/>
+      <x:c r="O12" s="63" t="str">
+        <x:v>DBM manual pp. 178–179 (PDF pp. 193–194)</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="57" t="str">
@@ -4511,7 +4729,9 @@
       <x:c r="N13" s="57" t="str">
         <x:v>MAP-008</x:v>
       </x:c>
-      <x:c r="O13" s="63" t="str"/>
+      <x:c r="O13" s="63" t="str">
+        <x:v>DBM manual pp. 178–179 (PDF pp. 193–194)</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="57" t="str">
@@ -4550,7 +4770,9 @@
       <x:c r="N14" s="57" t="str">
         <x:v>MAP-009</x:v>
       </x:c>
-      <x:c r="O14" s="63" t="str"/>
+      <x:c r="O14" s="63" t="str">
+        <x:v>DBM manual pp. 178–179 (PDF pp. 193–194)</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="57" t="str">
@@ -4589,7 +4811,9 @@
       <x:c r="N15" s="57" t="str">
         <x:v>MAP-010</x:v>
       </x:c>
-      <x:c r="O15" s="63" t="str"/>
+      <x:c r="O15" s="63" t="str">
+        <x:v>DBM manual pp. 205 (PDF pp. 220)</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="57" t="str">
@@ -4628,7 +4852,9 @@
       <x:c r="N16" s="57" t="str">
         <x:v>MAP-011</x:v>
       </x:c>
-      <x:c r="O16" s="63" t="str"/>
+      <x:c r="O16" s="63" t="str">
+        <x:v>DBM manual pp. 205 (PDF pp. 220)</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="57" t="str">
@@ -4667,7 +4893,9 @@
       <x:c r="N17" s="57" t="str">
         <x:v>MAP-012</x:v>
       </x:c>
-      <x:c r="O17" s="63" t="str"/>
+      <x:c r="O17" s="63" t="str">
+        <x:v>DBM manual pp. 205 (PDF pp. 220)</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="57" t="str">
@@ -4706,7 +4934,9 @@
       <x:c r="N18" s="57" t="str">
         <x:v>MAP-013</x:v>
       </x:c>
-      <x:c r="O18" s="63" t="str"/>
+      <x:c r="O18" s="63" t="str">
+        <x:v>DBM manual pp. 205 (PDF pp. 220)</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="57" t="str">
@@ -4745,7 +4975,9 @@
       <x:c r="N19" s="57" t="str">
         <x:v>MAP-014</x:v>
       </x:c>
-      <x:c r="O19" s="63" t="str"/>
+      <x:c r="O19" s="63" t="str">
+        <x:v>DBM manual pp. 206–207 (PDF pp. 221–222)</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="57" t="str">
@@ -4784,7 +5016,9 @@
       <x:c r="N20" s="57" t="str">
         <x:v>MAP-015</x:v>
       </x:c>
-      <x:c r="O20" s="63" t="str"/>
+      <x:c r="O20" s="63" t="str">
+        <x:v>DBM manual pp. 206–207 (PDF pp. 221–222)</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="57" t="str">
@@ -4823,7 +5057,9 @@
       <x:c r="N21" s="57" t="str">
         <x:v>MAP-016</x:v>
       </x:c>
-      <x:c r="O21" s="63" t="str"/>
+      <x:c r="O21" s="63" t="str">
+        <x:v>DBM manual pp. 206–207 (PDF pp. 221–222)</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="57" t="str">
@@ -4862,7 +5098,9 @@
       <x:c r="N22" s="57" t="str">
         <x:v>MAP-017</x:v>
       </x:c>
-      <x:c r="O22" s="63" t="str"/>
+      <x:c r="O22" s="63" t="str">
+        <x:v>DBM manual pp. 208 (PDF pp. 223)</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="57" t="str">
@@ -4901,7 +5139,9 @@
       <x:c r="N23" s="57" t="str">
         <x:v>MAP-018</x:v>
       </x:c>
-      <x:c r="O23" s="63" t="str"/>
+      <x:c r="O23" s="63" t="str">
+        <x:v>DBM manual pp. 208 (PDF pp. 223)</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="57" t="str">
@@ -4940,7 +5180,9 @@
       <x:c r="N24" s="57" t="str">
         <x:v>MAP-019</x:v>
       </x:c>
-      <x:c r="O24" s="63" t="str"/>
+      <x:c r="O24" s="63" t="str">
+        <x:v>DBM manual pp. 209–210 (PDF pp. 224–225)</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="57" t="str">
@@ -4979,7 +5221,9 @@
       <x:c r="N25" s="57" t="str">
         <x:v>MAP-020</x:v>
       </x:c>
-      <x:c r="O25" s="63" t="str"/>
+      <x:c r="O25" s="63" t="str">
+        <x:v>DBM manual pp. 209–210 (PDF pp. 224–225)</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="57" t="str">
@@ -5018,7 +5262,9 @@
       <x:c r="N26" s="57" t="str">
         <x:v>MAP-021</x:v>
       </x:c>
-      <x:c r="O26" s="63" t="str"/>
+      <x:c r="O26" s="63" t="str">
+        <x:v>DBM manual pp. 209–210 (PDF pp. 224–225)</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="57" t="str">
@@ -5057,7 +5303,9 @@
       <x:c r="N27" s="57" t="str">
         <x:v>MAP-022</x:v>
       </x:c>
-      <x:c r="O27" s="63" t="str"/>
+      <x:c r="O27" s="63" t="str">
+        <x:v>DBM manual pp. 211 (PDF pp. 226)</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="57" t="str">
@@ -5096,7 +5344,9 @@
       <x:c r="N28" s="57" t="str">
         <x:v>MAP-023</x:v>
       </x:c>
-      <x:c r="O28" s="63" t="str"/>
+      <x:c r="O28" s="63" t="str">
+        <x:v>DBM manual pp. 211 (PDF pp. 226)</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="57" t="str">
@@ -5135,53 +5385,1902 @@
       <x:c r="N29" s="57" t="str">
         <x:v>MAP-024</x:v>
       </x:c>
-      <x:c r="O29" s="63" t="str"/>
+      <x:c r="O29" s="63" t="str">
+        <x:v>DBM manual pp. 212–213 (PDF pp. 227–228)</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="58" t="str">
+      <x:c r="A30" s="57" t="str">
         <x:v>LBAc Form 6</x:v>
       </x:c>
-      <x:c r="B30" s="58" t="str">
+      <x:c r="B30" s="57" t="str">
         <x:v>Repeating table</x:v>
       </x:c>
-      <x:c r="C30" s="58" t="str">
+      <x:c r="C30" s="57" t="str">
         <x:v>Actual accomplishment; AIP/AB estimate; actual expenditures; remarks</x:v>
       </x:c>
-      <x:c r="D30" s="58" t="str">
+      <x:c r="D30" s="57" t="str">
         <x:v>Repeating</x:v>
       </x:c>
-      <x:c r="E30" s="58" t="str">
+      <x:c r="E30" s="57" t="str">
         <x:v>Accomplishment evidence and posted ledger</x:v>
       </x:c>
-      <x:c r="F30" s="58" t="str">
+      <x:c r="F30" s="57" t="str">
         <x:v>Link evidence without copying confidential files</x:v>
       </x:c>
-      <x:c r="G30" s="58" t="str">
+      <x:c r="G30" s="57" t="str">
         <x:v>Amounts and accomplishments tie to sources</x:v>
       </x:c>
-      <x:c r="H30" s="58" t="str">
+      <x:c r="H30" s="57" t="str">
         <x:v>Department / Budget / Accounting</x:v>
       </x:c>
-      <x:c r="I30" s="58" t="str">
+      <x:c r="I30" s="57" t="str">
         <x:v>Readable remarks</x:v>
       </x:c>
-      <x:c r="J30" s="64" t="str">
+      <x:c r="J30" s="63" t="str">
         <x:v>Starter - verify</x:v>
       </x:c>
-      <x:c r="K30" s="64" t="str"/>
-      <x:c r="L30" s="64" t="str"/>
-      <x:c r="M30" s="64" t="str"/>
-      <x:c r="N30" s="58" t="str">
+      <x:c r="K30" s="63" t="str"/>
+      <x:c r="L30" s="63" t="str"/>
+      <x:c r="M30" s="63" t="str"/>
+      <x:c r="N30" s="57" t="str">
         <x:v>MAP-025</x:v>
       </x:c>
-      <x:c r="O30" s="64" t="str"/>
+      <x:c r="O30" s="63" t="str">
+        <x:v>DBM manual pp. 212–213 (PDF pp. 227–228)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="57" t="str">
+        <x:v>LBP Form 1</x:v>
+      </x:c>
+      <x:c r="B31" s="57" t="str">
+        <x:v>Header</x:v>
+      </x:c>
+      <x:c r="C31" s="57" t="str">
+        <x:v>LGU; fund; budget year; past/current/budget-year period labels</x:v>
+      </x:c>
+      <x:c r="D31" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E31" s="57" t="str">
+        <x:v>Finance Setup and annual budget cycle</x:v>
+      </x:c>
+      <x:c r="F31" s="57" t="str">
+        <x:v>Pin fiscal year, fund, LGU, and comparison periods</x:v>
+      </x:c>
+      <x:c r="G31" s="57" t="str">
+        <x:v>All columns use the same approved period basis</x:v>
+      </x:c>
+      <x:c r="H31" s="57" t="str">
+        <x:v>Local Finance Committee / Accounting</x:v>
+      </x:c>
+      <x:c r="I31" s="57" t="str">
+        <x:v>Repeat identity and period headings</x:v>
+      </x:c>
+      <x:c r="J31" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K31" s="63" t="str"/>
+      <x:c r="L31" s="63" t="str"/>
+      <x:c r="M31" s="63" t="str"/>
+      <x:c r="N31" s="57" t="str">
+        <x:v>MAP-026</x:v>
+      </x:c>
+      <x:c r="O31" s="63" t="str">
+        <x:v>DBM manual pp. 59–61 (PDF pp. 74–76)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="57" t="str">
+        <x:v>LBP Form 1</x:v>
+      </x:c>
+      <x:c r="B32" s="57" t="str">
+        <x:v>Receipts program</x:v>
+      </x:c>
+      <x:c r="C32" s="57" t="str">
+        <x:v>Beginning cash; regular/non-regular income; local/external sources; financing</x:v>
+      </x:c>
+      <x:c r="D32" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E32" s="57" t="str">
+        <x:v>Approved resource estimates and posted historical receipts</x:v>
+      </x:c>
+      <x:c r="F32" s="57" t="str">
+        <x:v>Map accepted RCA-LGU income accounts and funding-source classes</x:v>
+      </x:c>
+      <x:c r="G32" s="57" t="str">
+        <x:v>Section subtotals and total available resources cross-foot</x:v>
+      </x:c>
+      <x:c r="H32" s="57" t="str">
+        <x:v>Treasury / Accounting / Budget</x:v>
+      </x:c>
+      <x:c r="I32" s="57" t="str">
+        <x:v>Repeat headings and preserve hierarchy</x:v>
+      </x:c>
+      <x:c r="J32" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K32" s="63" t="str"/>
+      <x:c r="L32" s="63" t="str"/>
+      <x:c r="M32" s="63" t="str"/>
+      <x:c r="N32" s="57" t="str">
+        <x:v>MAP-027</x:v>
+      </x:c>
+      <x:c r="O32" s="63" t="str">
+        <x:v>DBM manual pp. 59–61 (PDF pp. 74–76)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="57" t="str">
+        <x:v>LBP Form 1</x:v>
+      </x:c>
+      <x:c r="B33" s="57" t="str">
+        <x:v>Expenditure and financing</x:v>
+      </x:c>
+      <x:c r="C33" s="57" t="str">
+        <x:v>Expense class/object; debt/financing; surplus or deficit; certification</x:v>
+      </x:c>
+      <x:c r="D33" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E33" s="57" t="str">
+        <x:v>Department proposals, debt records, and financing plan</x:v>
+      </x:c>
+      <x:c r="F33" s="57" t="str">
+        <x:v>Preserve accepted sign and account presentation</x:v>
+      </x:c>
+      <x:c r="G33" s="57" t="str">
+        <x:v>Expenditures, financing, and budget balance reconcile</x:v>
+      </x:c>
+      <x:c r="H33" s="57" t="str">
+        <x:v>Local Finance Committee / Accounting / LCE</x:v>
+      </x:c>
+      <x:c r="I33" s="57" t="str">
+        <x:v>Accounting format; retain signature space</x:v>
+      </x:c>
+      <x:c r="J33" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K33" s="63" t="str"/>
+      <x:c r="L33" s="63" t="str"/>
+      <x:c r="M33" s="63" t="str"/>
+      <x:c r="N33" s="57" t="str">
+        <x:v>MAP-028</x:v>
+      </x:c>
+      <x:c r="O33" s="63" t="str">
+        <x:v>DBM manual pp. 59–61 (PDF pp. 74–76)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="57" t="str">
+        <x:v>LBP Form 2</x:v>
+      </x:c>
+      <x:c r="B34" s="57" t="str">
+        <x:v>Header and rows</x:v>
+      </x:c>
+      <x:c r="C34" s="57" t="str">
+        <x:v>LGU; department; object of expenditure; account code; comparison periods</x:v>
+      </x:c>
+      <x:c r="D34" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E34" s="57" t="str">
+        <x:v>Department proposal and posted historical expenses</x:v>
+      </x:c>
+      <x:c r="F34" s="57" t="str">
+        <x:v>Map exact accepted expense classifications</x:v>
+      </x:c>
+      <x:c r="G34" s="57" t="str">
+        <x:v>Past/current/proposed period columns use one basis</x:v>
+      </x:c>
+      <x:c r="H34" s="57" t="str">
+        <x:v>Department / Budget</x:v>
+      </x:c>
+      <x:c r="I34" s="57" t="str">
+        <x:v>Repeat headings and expense-class hierarchy</x:v>
+      </x:c>
+      <x:c r="J34" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K34" s="63" t="str"/>
+      <x:c r="L34" s="63" t="str"/>
+      <x:c r="M34" s="63" t="str"/>
+      <x:c r="N34" s="57" t="str">
+        <x:v>MAP-029</x:v>
+      </x:c>
+      <x:c r="O34" s="63" t="str">
+        <x:v>DBM manual pp. 62–63 (PDF pp. 77–78)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="57" t="str">
+        <x:v>LBP Form 2</x:v>
+      </x:c>
+      <x:c r="B35" s="57" t="str">
+        <x:v>Totals and certification</x:v>
+      </x:c>
+      <x:c r="C35" s="57" t="str">
+        <x:v>PS; MOOE; FE; CO; special-purpose appropriations; total; signatures</x:v>
+      </x:c>
+      <x:c r="D35" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E35" s="57" t="str">
+        <x:v>Classified proposal totals and wet-signature route</x:v>
+      </x:c>
+      <x:c r="F35" s="57" t="str">
+        <x:v>Roll up objects to accepted expense classes</x:v>
+      </x:c>
+      <x:c r="G35" s="57" t="str">
+        <x:v>All class totals reconcile to department proposal</x:v>
+      </x:c>
+      <x:c r="H35" s="57" t="str">
+        <x:v>Department Head / LBO / LCE</x:v>
+      </x:c>
+      <x:c r="I35" s="57" t="str">
+        <x:v>Retain totals and signature space</x:v>
+      </x:c>
+      <x:c r="J35" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K35" s="63" t="str"/>
+      <x:c r="L35" s="63" t="str"/>
+      <x:c r="M35" s="63" t="str"/>
+      <x:c r="N35" s="57" t="str">
+        <x:v>MAP-030</x:v>
+      </x:c>
+      <x:c r="O35" s="63" t="str">
+        <x:v>DBM manual pp. 62–63 (PDF pp. 77–78)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="57" t="str">
+        <x:v>LBP Form 3</x:v>
+      </x:c>
+      <x:c r="B36" s="57" t="str">
+        <x:v>Position identity</x:v>
+      </x:c>
+      <x:c r="C36" s="57" t="str">
+        <x:v>Old/new item number; position title; incumbent or vacancy</x:v>
+      </x:c>
+      <x:c r="D36" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E36" s="57" t="str">
+        <x:v>Approved personnel plantilla and HR records</x:v>
+      </x:c>
+      <x:c r="F36" s="57" t="str">
+        <x:v>Preserve vacancy, abolition, and reclassification notation</x:v>
+      </x:c>
+      <x:c r="G36" s="57" t="str">
+        <x:v>Every current/proposed item has a stable row identity</x:v>
+      </x:c>
+      <x:c r="H36" s="57" t="str">
+        <x:v>HRMO / Budget</x:v>
+      </x:c>
+      <x:c r="I36" s="57" t="str">
+        <x:v>Do not split one position across pages</x:v>
+      </x:c>
+      <x:c r="J36" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K36" s="63" t="str"/>
+      <x:c r="L36" s="63" t="str"/>
+      <x:c r="M36" s="63" t="str"/>
+      <x:c r="N36" s="57" t="str">
+        <x:v>MAP-031</x:v>
+      </x:c>
+      <x:c r="O36" s="63" t="str">
+        <x:v>DBM manual pp. 64–66 (PDF pp. 79–81)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="57" t="str">
+        <x:v>LBP Form 3</x:v>
+      </x:c>
+      <x:c r="B37" s="57" t="str">
+        <x:v>Salary comparison</x:v>
+      </x:c>
+      <x:c r="C37" s="57" t="str">
+        <x:v>Current authorized rate/amount; proposed SG/step/rate/amount; increase/decrease</x:v>
+      </x:c>
+      <x:c r="D37" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E37" s="57" t="str">
+        <x:v>Approved compensation schedule and proposed personnel services</x:v>
+      </x:c>
+      <x:c r="F37" s="57" t="str">
+        <x:v>Use locally accepted salary-grade and step mapping</x:v>
+      </x:c>
+      <x:c r="G37" s="57" t="str">
+        <x:v>Increase/decrease and total PS reconcile</x:v>
+      </x:c>
+      <x:c r="H37" s="57" t="str">
+        <x:v>HRMO / Budget</x:v>
+      </x:c>
+      <x:c r="I37" s="57" t="str">
+        <x:v>Currency/count formats and repeated headings</x:v>
+      </x:c>
+      <x:c r="J37" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K37" s="63" t="str"/>
+      <x:c r="L37" s="63" t="str"/>
+      <x:c r="M37" s="63" t="str"/>
+      <x:c r="N37" s="57" t="str">
+        <x:v>MAP-032</x:v>
+      </x:c>
+      <x:c r="O37" s="63" t="str">
+        <x:v>DBM manual pp. 64–66 (PDF pp. 79–81)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="57" t="str">
+        <x:v>LBP Form 3</x:v>
+      </x:c>
+      <x:c r="B38" s="57" t="str">
+        <x:v>Certification</x:v>
+      </x:c>
+      <x:c r="C38" s="57" t="str">
+        <x:v>Prepared; reviewed; approved names, titles, and signature dates</x:v>
+      </x:c>
+      <x:c r="D38" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E38" s="57" t="str">
+        <x:v>Wet-signature custody evidence</x:v>
+      </x:c>
+      <x:c r="F38" s="57" t="str">
+        <x:v>Use accepted local signatory route</x:v>
+      </x:c>
+      <x:c r="G38" s="57" t="str">
+        <x:v>Never imply digital signature</x:v>
+      </x:c>
+      <x:c r="H38" s="57" t="str">
+        <x:v>HRMO / LBO / LCE</x:v>
+      </x:c>
+      <x:c r="I38" s="57" t="str">
+        <x:v>Preserve signature space</x:v>
+      </x:c>
+      <x:c r="J38" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K38" s="63" t="str"/>
+      <x:c r="L38" s="63" t="str"/>
+      <x:c r="M38" s="63" t="str"/>
+      <x:c r="N38" s="57" t="str">
+        <x:v>MAP-033</x:v>
+      </x:c>
+      <x:c r="O38" s="63" t="str">
+        <x:v>DBM manual pp. 64–66 (PDF pp. 79–81)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="57" t="str">
+        <x:v>LBP Form 5</x:v>
+      </x:c>
+      <x:c r="B39" s="57" t="str">
+        <x:v>Debt schedule</x:v>
+      </x:c>
+      <x:c r="C39" s="57" t="str">
+        <x:v>Creditor; contract date; term; principal; purpose</x:v>
+      </x:c>
+      <x:c r="D39" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E39" s="57" t="str">
+        <x:v>Approved debt and contract register</x:v>
+      </x:c>
+      <x:c r="F39" s="57" t="str">
+        <x:v>One row per debt instrument/fund/special account</x:v>
+      </x:c>
+      <x:c r="G39" s="57" t="str">
+        <x:v>Principal and instrument identity agree with retained evidence</x:v>
+      </x:c>
+      <x:c r="H39" s="57" t="str">
+        <x:v>Accounting</x:v>
+      </x:c>
+      <x:c r="I39" s="57" t="str">
+        <x:v>Repeat headings; readable creditor/purpose</x:v>
+      </x:c>
+      <x:c r="J39" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K39" s="63" t="str"/>
+      <x:c r="L39" s="63" t="str"/>
+      <x:c r="M39" s="63" t="str"/>
+      <x:c r="N39" s="57" t="str">
+        <x:v>MAP-034</x:v>
+      </x:c>
+      <x:c r="O39" s="63" t="str">
+        <x:v>DBM manual pp. 67 (PDF pp. 82)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="57" t="str">
+        <x:v>LBP Form 5</x:v>
+      </x:c>
+      <x:c r="B40" s="57" t="str">
+        <x:v>Payments and balance</x:v>
+      </x:c>
+      <x:c r="C40" s="57" t="str">
+        <x:v>Previous principal/interest/total; amount due; ending principal balance; certification</x:v>
+      </x:c>
+      <x:c r="D40" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E40" s="57" t="str">
+        <x:v>Posted debt-service transactions and schedule</x:v>
+      </x:c>
+      <x:c r="F40" s="57" t="str">
+        <x:v>Calculate from accepted debt roll-forward</x:v>
+      </x:c>
+      <x:c r="G40" s="57" t="str">
+        <x:v>Opening principal less payments equals balance; due totals cross-foot</x:v>
+      </x:c>
+      <x:c r="H40" s="57" t="str">
+        <x:v>Local Accountant / LCE</x:v>
+      </x:c>
+      <x:c r="I40" s="57" t="str">
+        <x:v>Accounting format; signature space</x:v>
+      </x:c>
+      <x:c r="J40" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K40" s="63" t="str"/>
+      <x:c r="L40" s="63" t="str"/>
+      <x:c r="M40" s="63" t="str"/>
+      <x:c r="N40" s="57" t="str">
+        <x:v>MAP-035</x:v>
+      </x:c>
+      <x:c r="O40" s="63" t="str">
+        <x:v>DBM manual pp. 67 (PDF pp. 82)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="57" t="str">
+        <x:v>LBP Form 6</x:v>
+      </x:c>
+      <x:c r="B41" s="57" t="str">
+        <x:v>Requirement schedule</x:v>
+      </x:c>
+      <x:c r="C41" s="57" t="str">
+        <x:v>Statutory/contractual obligation or budgetary requirement; amount</x:v>
+      </x:c>
+      <x:c r="D41" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E41" s="57" t="str">
+        <x:v>Approved policy, contract, personnel, debt, and budget rules</x:v>
+      </x:c>
+      <x:c r="F41" s="57" t="str">
+        <x:v>Keep each locally applicable requirement separately identifiable</x:v>
+      </x:c>
+      <x:c r="G41" s="57" t="str">
+        <x:v>Section subtotals and overall total cross-foot</x:v>
+      </x:c>
+      <x:c r="H41" s="57" t="str">
+        <x:v>Local Finance Committee</x:v>
+      </x:c>
+      <x:c r="I41" s="57" t="str">
+        <x:v>Readable authority notes where locally required</x:v>
+      </x:c>
+      <x:c r="J41" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K41" s="63" t="str"/>
+      <x:c r="L41" s="63" t="str"/>
+      <x:c r="M41" s="63" t="str"/>
+      <x:c r="N41" s="57" t="str">
+        <x:v>MAP-036</x:v>
+      </x:c>
+      <x:c r="O41" s="63" t="str">
+        <x:v>DBM manual pp. 68 (PDF pp. 83)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="57" t="str">
+        <x:v>LBP Form 6</x:v>
+      </x:c>
+      <x:c r="B42" s="57" t="str">
+        <x:v>Certification</x:v>
+      </x:c>
+      <x:c r="C42" s="57" t="str">
+        <x:v>Budget Officer; Treasurer; Accountant certification; LCE approval</x:v>
+      </x:c>
+      <x:c r="D42" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E42" s="57" t="str">
+        <x:v>Wet-signature custody evidence</x:v>
+      </x:c>
+      <x:c r="F42" s="57" t="str">
+        <x:v>Use current local committee and approval route</x:v>
+      </x:c>
+      <x:c r="G42" s="57" t="str">
+        <x:v>Never imply digital signature</x:v>
+      </x:c>
+      <x:c r="H42" s="57" t="str">
+        <x:v>LFC / LCE</x:v>
+      </x:c>
+      <x:c r="I42" s="57" t="str">
+        <x:v>Preserve signature space</x:v>
+      </x:c>
+      <x:c r="J42" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K42" s="63" t="str"/>
+      <x:c r="L42" s="63" t="str"/>
+      <x:c r="M42" s="63" t="str"/>
+      <x:c r="N42" s="57" t="str">
+        <x:v>MAP-037</x:v>
+      </x:c>
+      <x:c r="O42" s="63" t="str">
+        <x:v>DBM manual pp. 68 (PDF pp. 83)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="57" t="str">
+        <x:v>LBP Form 7</x:v>
+      </x:c>
+      <x:c r="B43" s="57" t="str">
+        <x:v>Sector allocation</x:v>
+      </x:c>
+      <x:c r="C43" s="57" t="str">
+        <x:v>Particular; account code; General Public/Social/Economic/Other Services; total</x:v>
+      </x:c>
+      <x:c r="D43" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E43" s="57" t="str">
+        <x:v>Approved PPA and sector mapping</x:v>
+      </x:c>
+      <x:c r="F43" s="57" t="str">
+        <x:v>Use accepted sector and RCA-LGU mapping</x:v>
+      </x:c>
+      <x:c r="G43" s="57" t="str">
+        <x:v>Row total equals sector columns; sector totals equal appropriations</x:v>
+      </x:c>
+      <x:c r="H43" s="57" t="str">
+        <x:v>Budget</x:v>
+      </x:c>
+      <x:c r="I43" s="57" t="str">
+        <x:v>Repeat headings and sector labels</x:v>
+      </x:c>
+      <x:c r="J43" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K43" s="63" t="str"/>
+      <x:c r="L43" s="63" t="str"/>
+      <x:c r="M43" s="63" t="str"/>
+      <x:c r="N43" s="57" t="str">
+        <x:v>MAP-038</x:v>
+      </x:c>
+      <x:c r="O43" s="63" t="str">
+        <x:v>DBM manual pp. 69 (PDF pp. 84)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="57" t="str">
+        <x:v>LBP Form 7</x:v>
+      </x:c>
+      <x:c r="B44" s="57" t="str">
+        <x:v>Certification</x:v>
+      </x:c>
+      <x:c r="C44" s="57" t="str">
+        <x:v>Total appropriations; LBO certification; LCE approval</x:v>
+      </x:c>
+      <x:c r="D44" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E44" s="57" t="str">
+        <x:v>Approved annual budget and wet-signature evidence</x:v>
+      </x:c>
+      <x:c r="F44" s="57" t="str">
+        <x:v>Pin source budget version</x:v>
+      </x:c>
+      <x:c r="G44" s="57" t="str">
+        <x:v>Form total equals approved appropriation control</x:v>
+      </x:c>
+      <x:c r="H44" s="57" t="str">
+        <x:v>LBO / LCE</x:v>
+      </x:c>
+      <x:c r="I44" s="57" t="str">
+        <x:v>Accounting format; signature space</x:v>
+      </x:c>
+      <x:c r="J44" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K44" s="63" t="str"/>
+      <x:c r="L44" s="63" t="str"/>
+      <x:c r="M44" s="63" t="str"/>
+      <x:c r="N44" s="57" t="str">
+        <x:v>MAP-039</x:v>
+      </x:c>
+      <x:c r="O44" s="63" t="str">
+        <x:v>DBM manual pp. 69 (PDF pp. 84)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="57" t="str">
+        <x:v>LBP Form 8</x:v>
+      </x:c>
+      <x:c r="B45" s="57" t="str">
+        <x:v>Funding-source rows</x:v>
+      </x:c>
+      <x:c r="C45" s="57" t="str">
+        <x:v>Fund/special account; source particular; account classification; amount</x:v>
+      </x:c>
+      <x:c r="D45" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E45" s="57" t="str">
+        <x:v>Supplemental funding evidence and accepted classifications</x:v>
+      </x:c>
+      <x:c r="F45" s="57" t="str">
+        <x:v>Distinguish new revenue, excess collection, savings, and realignment</x:v>
+      </x:c>
+      <x:c r="G45" s="57" t="str">
+        <x:v>Source total equals available supplemental authority</x:v>
+      </x:c>
+      <x:c r="H45" s="57" t="str">
+        <x:v>Treasury / Accounting</x:v>
+      </x:c>
+      <x:c r="I45" s="57" t="str">
+        <x:v>Repeat headings; readable source detail</x:v>
+      </x:c>
+      <x:c r="J45" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K45" s="63" t="str"/>
+      <x:c r="L45" s="63" t="str"/>
+      <x:c r="M45" s="63" t="str"/>
+      <x:c r="N45" s="57" t="str">
+        <x:v>MAP-040</x:v>
+      </x:c>
+      <x:c r="O45" s="63" t="str">
+        <x:v>DBM manual pp. 70 (PDF pp. 85)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="57" t="str">
+        <x:v>LBP Form 8</x:v>
+      </x:c>
+      <x:c r="B46" s="57" t="str">
+        <x:v>Certification</x:v>
+      </x:c>
+      <x:c r="C46" s="57" t="str">
+        <x:v>Treasurer and/or Accountant certification by funding source</x:v>
+      </x:c>
+      <x:c r="D46" s="57" t="str">
+        <x:v>Conditional</x:v>
+      </x:c>
+      <x:c r="E46" s="57" t="str">
+        <x:v>Wet-signature custody and funding-source authority</x:v>
+      </x:c>
+      <x:c r="F46" s="57" t="str">
+        <x:v>Apply the locally confirmed signatory condition</x:v>
+      </x:c>
+      <x:c r="G46" s="57" t="str">
+        <x:v>Each source has required certification</x:v>
+      </x:c>
+      <x:c r="H46" s="57" t="str">
+        <x:v>Treasury / Accounting</x:v>
+      </x:c>
+      <x:c r="I46" s="57" t="str">
+        <x:v>Preserve conditional signature space</x:v>
+      </x:c>
+      <x:c r="J46" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K46" s="63" t="str"/>
+      <x:c r="L46" s="63" t="str"/>
+      <x:c r="M46" s="63" t="str"/>
+      <x:c r="N46" s="57" t="str">
+        <x:v>MAP-041</x:v>
+      </x:c>
+      <x:c r="O46" s="63" t="str">
+        <x:v>DBM manual pp. 70 (PDF pp. 85)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="57" t="str">
+        <x:v>LBP Form 9</x:v>
+      </x:c>
+      <x:c r="B47" s="57" t="str">
+        <x:v>Supplemental appropriation</x:v>
+      </x:c>
+      <x:c r="C47" s="57" t="str">
+        <x:v>Implementing office; purpose/PPA; AIP reference; object; account code; amount</x:v>
+      </x:c>
+      <x:c r="D47" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E47" s="57" t="str">
+        <x:v>Approved supplemental AIP and appropriation proposal</x:v>
+      </x:c>
+      <x:c r="F47" s="57" t="str">
+        <x:v>Map office, PPA, AIP, object, and account identities exactly</x:v>
+      </x:c>
+      <x:c r="G47" s="57" t="str">
+        <x:v>Amounts total to the certified supplemental source</x:v>
+      </x:c>
+      <x:c r="H47" s="57" t="str">
+        <x:v>Budget / implementing office</x:v>
+      </x:c>
+      <x:c r="I47" s="57" t="str">
+        <x:v>Repeat headings; do not split PPA rows</x:v>
+      </x:c>
+      <x:c r="J47" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K47" s="63" t="str"/>
+      <x:c r="L47" s="63" t="str"/>
+      <x:c r="M47" s="63" t="str"/>
+      <x:c r="N47" s="57" t="str">
+        <x:v>MAP-042</x:v>
+      </x:c>
+      <x:c r="O47" s="63" t="str">
+        <x:v>DBM manual pp. 71 (PDF pp. 86)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="57" t="str">
+        <x:v>LBP Form 9</x:v>
+      </x:c>
+      <x:c r="B48" s="57" t="str">
+        <x:v>Certification</x:v>
+      </x:c>
+      <x:c r="C48" s="57" t="str">
+        <x:v>Prepared by LBO; approved by LCE</x:v>
+      </x:c>
+      <x:c r="D48" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E48" s="57" t="str">
+        <x:v>Wet-signature custody evidence</x:v>
+      </x:c>
+      <x:c r="F48" s="57" t="str">
+        <x:v>Use accepted local route</x:v>
+      </x:c>
+      <x:c r="G48" s="57" t="str">
+        <x:v>Never imply digital signature</x:v>
+      </x:c>
+      <x:c r="H48" s="57" t="str">
+        <x:v>LBO / LCE</x:v>
+      </x:c>
+      <x:c r="I48" s="57" t="str">
+        <x:v>Preserve totals and signature space</x:v>
+      </x:c>
+      <x:c r="J48" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K48" s="63" t="str"/>
+      <x:c r="L48" s="63" t="str"/>
+      <x:c r="M48" s="63" t="str"/>
+      <x:c r="N48" s="57" t="str">
+        <x:v>MAP-043</x:v>
+      </x:c>
+      <x:c r="O48" s="63" t="str">
+        <x:v>DBM manual pp. 71 (PDF pp. 86)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="57" t="str">
+        <x:v>LBA Form 1A</x:v>
+      </x:c>
+      <x:c r="B49" s="57" t="str">
+        <x:v>Document checklist</x:v>
+      </x:c>
+      <x:c r="C49" s="57" t="str">
+        <x:v>Annual-budget document; required signatory; remarks</x:v>
+      </x:c>
+      <x:c r="D49" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E49" s="57" t="str">
+        <x:v>F10 form register and retained document references</x:v>
+      </x:c>
+      <x:c r="F49" s="57" t="str">
+        <x:v>One row per locally applicable annual-budget requirement</x:v>
+      </x:c>
+      <x:c r="G49" s="57" t="str">
+        <x:v>No required item may be marked complete without exact evidence</x:v>
+      </x:c>
+      <x:c r="H49" s="57" t="str">
+        <x:v>Budget / Sanggunian records</x:v>
+      </x:c>
+      <x:c r="I49" s="57" t="str">
+        <x:v>Readable checklist; continuation allowed</x:v>
+      </x:c>
+      <x:c r="J49" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K49" s="63" t="str"/>
+      <x:c r="L49" s="63" t="str"/>
+      <x:c r="M49" s="63" t="str"/>
+      <x:c r="N49" s="57" t="str">
+        <x:v>MAP-044</x:v>
+      </x:c>
+      <x:c r="O49" s="63" t="str">
+        <x:v>DBM manual pp. 109 (PDF pp. 124)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="57" t="str">
+        <x:v>LBA Form 1A</x:v>
+      </x:c>
+      <x:c r="B50" s="57" t="str">
+        <x:v>Conditional documents</x:v>
+      </x:c>
+      <x:c r="C50" s="57" t="str">
+        <x:v>AIP/resolution; operating budget of local economic enterprise; other conditional items</x:v>
+      </x:c>
+      <x:c r="D50" s="57" t="str">
+        <x:v>Conditional</x:v>
+      </x:c>
+      <x:c r="E50" s="57" t="str">
+        <x:v>Annual-budget package profile and local decisions</x:v>
+      </x:c>
+      <x:c r="F50" s="57" t="str">
+        <x:v>Show condition and responsible signatory explicitly</x:v>
+      </x:c>
+      <x:c r="G50" s="57" t="str">
+        <x:v>Conditional item is either satisfied or documented not applicable</x:v>
+      </x:c>
+      <x:c r="H50" s="57" t="str">
+        <x:v>Budget / LPDO / LEE / Sanggunian</x:v>
+      </x:c>
+      <x:c r="I50" s="57" t="str">
+        <x:v>Keep remarks with the related item</x:v>
+      </x:c>
+      <x:c r="J50" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K50" s="63" t="str"/>
+      <x:c r="L50" s="63" t="str"/>
+      <x:c r="M50" s="63" t="str"/>
+      <x:c r="N50" s="57" t="str">
+        <x:v>MAP-045</x:v>
+      </x:c>
+      <x:c r="O50" s="63" t="str">
+        <x:v>DBM manual pp. 109 (PDF pp. 124)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="57" t="str">
+        <x:v>LBA Form 1B</x:v>
+      </x:c>
+      <x:c r="B51" s="57" t="str">
+        <x:v>Funding documents</x:v>
+      </x:c>
+      <x:c r="C51" s="57" t="str">
+        <x:v>Additional realized income; savings/reversion; new revenue measures and supporting authority</x:v>
+      </x:c>
+      <x:c r="D51" s="57" t="str">
+        <x:v>Conditional</x:v>
+      </x:c>
+      <x:c r="E51" s="57" t="str">
+        <x:v>Supplemental funding evidence and authority decisions</x:v>
+      </x:c>
+      <x:c r="F51" s="57" t="str">
+        <x:v>Select only the applicable source route</x:v>
+      </x:c>
+      <x:c r="G51" s="57" t="str">
+        <x:v>Certified funding sources equal proposed supplemental appropriation</x:v>
+      </x:c>
+      <x:c r="H51" s="57" t="str">
+        <x:v>Treasury / Accounting / Sanggunian</x:v>
+      </x:c>
+      <x:c r="I51" s="57" t="str">
+        <x:v>Continuation allowed; preserve signatories</x:v>
+      </x:c>
+      <x:c r="J51" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K51" s="63" t="str"/>
+      <x:c r="L51" s="63" t="str"/>
+      <x:c r="M51" s="63" t="str"/>
+      <x:c r="N51" s="57" t="str">
+        <x:v>MAP-046</x:v>
+      </x:c>
+      <x:c r="O51" s="63" t="str">
+        <x:v>DBM manual pp. 110–111 (PDF pp. 125–126)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="57" t="str">
+        <x:v>LBA Form 1B</x:v>
+      </x:c>
+      <x:c r="B52" s="57" t="str">
+        <x:v>Supplemental AIP and approval</x:v>
+      </x:c>
+      <x:c r="C52" s="57" t="str">
+        <x:v>Supplemental AIP; approving resolution; signatories; remarks</x:v>
+      </x:c>
+      <x:c r="D52" s="57" t="str">
+        <x:v>Conditional</x:v>
+      </x:c>
+      <x:c r="E52" s="57" t="str">
+        <x:v>Supplemental AIP and enacted authority evidence</x:v>
+      </x:c>
+      <x:c r="F52" s="57" t="str">
+        <x:v>Pin exact resolution and package version</x:v>
+      </x:c>
+      <x:c r="G52" s="57" t="str">
+        <x:v>Every locally required signature and document is resolved</x:v>
+      </x:c>
+      <x:c r="H52" s="57" t="str">
+        <x:v>LPDO / LBO / Sanggunian / LCE</x:v>
+      </x:c>
+      <x:c r="I52" s="57" t="str">
+        <x:v>Readable checklist and signature labels</x:v>
+      </x:c>
+      <x:c r="J52" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K52" s="63" t="str"/>
+      <x:c r="L52" s="63" t="str"/>
+      <x:c r="M52" s="63" t="str"/>
+      <x:c r="N52" s="57" t="str">
+        <x:v>MAP-047</x:v>
+      </x:c>
+      <x:c r="O52" s="63" t="str">
+        <x:v>DBM manual pp. 110–111 (PDF pp. 125–126)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="57" t="str">
+        <x:v>LBR Form 1A</x:v>
+      </x:c>
+      <x:c r="B53" s="57" t="str">
+        <x:v>Review identity</x:v>
+      </x:c>
+      <x:c r="C53" s="57" t="str">
+        <x:v>Date received; deadline; LGU; class; title; fund</x:v>
+      </x:c>
+      <x:c r="D53" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E53" s="57" t="str">
+        <x:v>Budget-review submission and calendar</x:v>
+      </x:c>
+      <x:c r="F53" s="57" t="str">
+        <x:v>Pin received package and statutory/local deadline</x:v>
+      </x:c>
+      <x:c r="G53" s="57" t="str">
+        <x:v>Deadline derives from accepted authority, not workbook assumption</x:v>
+      </x:c>
+      <x:c r="H53" s="57" t="str">
+        <x:v>Reviewing authority</x:v>
+      </x:c>
+      <x:c r="I53" s="57" t="str">
+        <x:v>Keep identity on continuation pages</x:v>
+      </x:c>
+      <x:c r="J53" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K53" s="63" t="str"/>
+      <x:c r="L53" s="63" t="str"/>
+      <x:c r="M53" s="63" t="str"/>
+      <x:c r="N53" s="57" t="str">
+        <x:v>MAP-048</x:v>
+      </x:c>
+      <x:c r="O53" s="63" t="str">
+        <x:v>DBM manual pp. 136 (PDF pp. 151)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="57" t="str">
+        <x:v>LBR Form 1A</x:v>
+      </x:c>
+      <x:c r="B54" s="57" t="str">
+        <x:v>Annual review checklist</x:v>
+      </x:c>
+      <x:c r="C54" s="57" t="str">
+        <x:v>Transmittal, message, ordinance, AIP, supporting documents, signatories, remarks</x:v>
+      </x:c>
+      <x:c r="D54" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E54" s="57" t="str">
+        <x:v>Submitted annual-budget package</x:v>
+      </x:c>
+      <x:c r="F54" s="57" t="str">
+        <x:v>One row per current documentary/signature requirement</x:v>
+      </x:c>
+      <x:c r="G54" s="57" t="str">
+        <x:v>Missing or inconsistent items remain visible</x:v>
+      </x:c>
+      <x:c r="H54" s="57" t="str">
+        <x:v>Reviewing officer</x:v>
+      </x:c>
+      <x:c r="I54" s="57" t="str">
+        <x:v>Repeat headings; readable remarks</x:v>
+      </x:c>
+      <x:c r="J54" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K54" s="63" t="str"/>
+      <x:c r="L54" s="63" t="str"/>
+      <x:c r="M54" s="63" t="str"/>
+      <x:c r="N54" s="57" t="str">
+        <x:v>MAP-049</x:v>
+      </x:c>
+      <x:c r="O54" s="63" t="str">
+        <x:v>DBM manual pp. 136 (PDF pp. 151)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="57" t="str">
+        <x:v>LBR Form 1B</x:v>
+      </x:c>
+      <x:c r="B55" s="57" t="str">
+        <x:v>Review identity</x:v>
+      </x:c>
+      <x:c r="C55" s="57" t="str">
+        <x:v>Date received; deadline; LGU; class; title; fund</x:v>
+      </x:c>
+      <x:c r="D55" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E55" s="57" t="str">
+        <x:v>Supplemental-budget review submission and calendar</x:v>
+      </x:c>
+      <x:c r="F55" s="57" t="str">
+        <x:v>Pin received package and deadline basis</x:v>
+      </x:c>
+      <x:c r="G55" s="57" t="str">
+        <x:v>Deadline derives from accepted authority</x:v>
+      </x:c>
+      <x:c r="H55" s="57" t="str">
+        <x:v>Reviewing authority</x:v>
+      </x:c>
+      <x:c r="I55" s="57" t="str">
+        <x:v>Keep identity on continuation pages</x:v>
+      </x:c>
+      <x:c r="J55" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K55" s="63" t="str"/>
+      <x:c r="L55" s="63" t="str"/>
+      <x:c r="M55" s="63" t="str"/>
+      <x:c r="N55" s="57" t="str">
+        <x:v>MAP-050</x:v>
+      </x:c>
+      <x:c r="O55" s="63" t="str">
+        <x:v>DBM manual pp. 137–138 (PDF pp. 152–153)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="57" t="str">
+        <x:v>LBR Form 1B</x:v>
+      </x:c>
+      <x:c r="B56" s="57" t="str">
+        <x:v>Supplemental review checklist</x:v>
+      </x:c>
+      <x:c r="C56" s="57" t="str">
+        <x:v>Transmittal; ordinance; funds available; new revenue; realignment/calamity; signatories</x:v>
+      </x:c>
+      <x:c r="D56" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E56" s="57" t="str">
+        <x:v>Submitted supplemental-budget package</x:v>
+      </x:c>
+      <x:c r="F56" s="57" t="str">
+        <x:v>Apply exact condition for each funding/realignment route</x:v>
+      </x:c>
+      <x:c r="G56" s="57" t="str">
+        <x:v>Every required item is evidenced or documented not applicable</x:v>
+      </x:c>
+      <x:c r="H56" s="57" t="str">
+        <x:v>Reviewing officer</x:v>
+      </x:c>
+      <x:c r="I56" s="57" t="str">
+        <x:v>Repeat headings; readable remarks</x:v>
+      </x:c>
+      <x:c r="J56" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K56" s="63" t="str"/>
+      <x:c r="L56" s="63" t="str"/>
+      <x:c r="M56" s="63" t="str"/>
+      <x:c r="N56" s="57" t="str">
+        <x:v>MAP-051</x:v>
+      </x:c>
+      <x:c r="O56" s="63" t="str">
+        <x:v>DBM manual pp. 137–138 (PDF pp. 152–153)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="57" t="str">
+        <x:v>LBR Form 2</x:v>
+      </x:c>
+      <x:c r="B57" s="57" t="str">
+        <x:v>Review identity</x:v>
+      </x:c>
+      <x:c r="C57" s="57" t="str">
+        <x:v>LGU; budget title; appropriation ordinance and reviewed amount references</x:v>
+      </x:c>
+      <x:c r="D57" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E57" s="57" t="str">
+        <x:v>Review submission and enacted budget evidence</x:v>
+      </x:c>
+      <x:c r="F57" s="57" t="str">
+        <x:v>Pin exact package and authority version</x:v>
+      </x:c>
+      <x:c r="G57" s="57" t="str">
+        <x:v>Identity agrees with LBR checklist</x:v>
+      </x:c>
+      <x:c r="H57" s="57" t="str">
+        <x:v>Reviewing officer</x:v>
+      </x:c>
+      <x:c r="I57" s="57" t="str">
+        <x:v>Repeat identity across multi-page form</x:v>
+      </x:c>
+      <x:c r="J57" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K57" s="63" t="str"/>
+      <x:c r="L57" s="63" t="str"/>
+      <x:c r="M57" s="63" t="str"/>
+      <x:c r="N57" s="57" t="str">
+        <x:v>MAP-052</x:v>
+      </x:c>
+      <x:c r="O57" s="63" t="str">
+        <x:v>DBM manual pp. 139–152 (PDF pp. 154–167)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="57" t="str">
+        <x:v>LBR Form 2</x:v>
+      </x:c>
+      <x:c r="B58" s="57" t="str">
+        <x:v>Findings</x:v>
+      </x:c>
+      <x:c r="C58" s="57" t="str">
+        <x:v>Finding; compliant yes/no; recommended review action</x:v>
+      </x:c>
+      <x:c r="D58" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E58" s="57" t="str">
+        <x:v>Applicable review policies and submitted evidence</x:v>
+      </x:c>
+      <x:c r="F58" s="57" t="str">
+        <x:v>Keep each finding and its authority separately reviewable</x:v>
+      </x:c>
+      <x:c r="G58" s="57" t="str">
+        <x:v>Every applicable finding has one decision and action</x:v>
+      </x:c>
+      <x:c r="H58" s="57" t="str">
+        <x:v>Reviewing officer / subject reviewer</x:v>
+      </x:c>
+      <x:c r="I58" s="57" t="str">
+        <x:v>Repeat headings across long form</x:v>
+      </x:c>
+      <x:c r="J58" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K58" s="63" t="str"/>
+      <x:c r="L58" s="63" t="str"/>
+      <x:c r="M58" s="63" t="str"/>
+      <x:c r="N58" s="57" t="str">
+        <x:v>MAP-053</x:v>
+      </x:c>
+      <x:c r="O58" s="63" t="str">
+        <x:v>DBM manual pp. 139–152 (PDF pp. 154–167)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="57" t="str">
+        <x:v>LBR Form 2</x:v>
+      </x:c>
+      <x:c r="B59" s="57" t="str">
+        <x:v>Overall review action</x:v>
+      </x:c>
+      <x:c r="C59" s="57" t="str">
+        <x:v>Operative/inoperative decision; conditions; prepared/reviewed/approved</x:v>
+      </x:c>
+      <x:c r="D59" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E59" s="57" t="str">
+        <x:v>Completed findings and wet-signature evidence</x:v>
+      </x:c>
+      <x:c r="F59" s="57" t="str">
+        <x:v>Allow only locally authorized overall outcomes</x:v>
+      </x:c>
+      <x:c r="G59" s="57" t="str">
+        <x:v>Overall action agrees with unresolved findings</x:v>
+      </x:c>
+      <x:c r="H59" s="57" t="str">
+        <x:v>Reviewing and approving authorities</x:v>
+      </x:c>
+      <x:c r="I59" s="57" t="str">
+        <x:v>Preserve decision and signature space</x:v>
+      </x:c>
+      <x:c r="J59" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K59" s="63" t="str"/>
+      <x:c r="L59" s="63" t="str"/>
+      <x:c r="M59" s="63" t="str"/>
+      <x:c r="N59" s="57" t="str">
+        <x:v>MAP-054</x:v>
+      </x:c>
+      <x:c r="O59" s="63" t="str">
+        <x:v>DBM manual pp. 139–152 (PDF pp. 154–167)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="57" t="str">
+        <x:v>LBR Form 2A</x:v>
+      </x:c>
+      <x:c r="B60" s="57" t="str">
+        <x:v>Waived PS costs</x:v>
+      </x:c>
+      <x:c r="C60" s="57" t="str">
+        <x:v>Transferred hospital-service items and other permitted waived PS components</x:v>
+      </x:c>
+      <x:c r="D60" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E60" s="57" t="str">
+        <x:v>Personnel budget and accepted waiver authority</x:v>
+      </x:c>
+      <x:c r="F60" s="57" t="str">
+        <x:v>Itemize each applicable salary, benefit, and contribution</x:v>
+      </x:c>
+      <x:c r="G60" s="57" t="str">
+        <x:v>Subtotals and total waived PS cost cross-foot</x:v>
+      </x:c>
+      <x:c r="H60" s="57" t="str">
+        <x:v>Budget reviewer / HR / Accounting</x:v>
+      </x:c>
+      <x:c r="I60" s="57" t="str">
+        <x:v>Preserve item hierarchy</x:v>
+      </x:c>
+      <x:c r="J60" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K60" s="63" t="str"/>
+      <x:c r="L60" s="63" t="str"/>
+      <x:c r="M60" s="63" t="str"/>
+      <x:c r="N60" s="57" t="str">
+        <x:v>MAP-055</x:v>
+      </x:c>
+      <x:c r="O60" s="63" t="str">
+        <x:v>DBM manual pp. 153 (PDF pp. 168)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="57" t="str">
+        <x:v>LBR Form 2A</x:v>
+      </x:c>
+      <x:c r="B61" s="57" t="str">
+        <x:v>Authority and total</x:v>
+      </x:c>
+      <x:c r="C61" s="57" t="str">
+        <x:v>Waiver basis; LGU; subtotal/total; reviewer evidence</x:v>
+      </x:c>
+      <x:c r="D61" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E61" s="57" t="str">
+        <x:v>Applicable waiver decision and review evidence</x:v>
+      </x:c>
+      <x:c r="F61" s="57" t="str">
+        <x:v>Do not treat a candidate waiver as approved</x:v>
+      </x:c>
+      <x:c r="G61" s="57" t="str">
+        <x:v>Only authority-backed amounts enter the total</x:v>
+      </x:c>
+      <x:c r="H61" s="57" t="str">
+        <x:v>Reviewing authority</x:v>
+      </x:c>
+      <x:c r="I61" s="57" t="str">
+        <x:v>Readable authority reference and total</x:v>
+      </x:c>
+      <x:c r="J61" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K61" s="63" t="str"/>
+      <x:c r="L61" s="63" t="str"/>
+      <x:c r="M61" s="63" t="str"/>
+      <x:c r="N61" s="57" t="str">
+        <x:v>MAP-056</x:v>
+      </x:c>
+      <x:c r="O61" s="63" t="str">
+        <x:v>DBM manual pp. 153 (PDF pp. 168)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="57" t="str">
+        <x:v>LBR Form 2B</x:v>
+      </x:c>
+      <x:c r="B62" s="57" t="str">
+        <x:v>Income and limit</x:v>
+      </x:c>
+      <x:c r="C62" s="57" t="str">
+        <x:v>TIRS; applicable 45%/55% factor; calculated PS limitation</x:v>
+      </x:c>
+      <x:c r="D62" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E62" s="57" t="str">
+        <x:v>Posted preceding-year regular income and accepted LGU classification</x:v>
+      </x:c>
+      <x:c r="F62" s="57" t="str">
+        <x:v>Keep factor as an explicit locally confirmed input</x:v>
+      </x:c>
+      <x:c r="G62" s="57" t="str">
+        <x:v>PS limit equals confirmed factor times TIRS</x:v>
+      </x:c>
+      <x:c r="H62" s="57" t="str">
+        <x:v>Budget review / Accounting</x:v>
+      </x:c>
+      <x:c r="I62" s="57" t="str">
+        <x:v>Percentage and currency formats</x:v>
+      </x:c>
+      <x:c r="J62" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K62" s="63" t="str"/>
+      <x:c r="L62" s="63" t="str"/>
+      <x:c r="M62" s="63" t="str"/>
+      <x:c r="N62" s="57" t="str">
+        <x:v>MAP-057</x:v>
+      </x:c>
+      <x:c r="O62" s="63" t="str">
+        <x:v>DBM manual pp. 154 (PDF pp. 169)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="57" t="str">
+        <x:v>LBR Form 2B</x:v>
+      </x:c>
+      <x:c r="B63" s="57" t="str">
+        <x:v>PS cost components</x:v>
+      </x:c>
+      <x:c r="C63" s="57" t="str">
+        <x:v>Existing/new positions; salaries; compensation; benefits; contributions; other authorized items</x:v>
+      </x:c>
+      <x:c r="D63" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E63" s="57" t="str">
+        <x:v>Plantilla and personnel-services proposal</x:v>
+      </x:c>
+      <x:c r="F63" s="57" t="str">
+        <x:v>Map every included/excluded component to authority</x:v>
+      </x:c>
+      <x:c r="G63" s="57" t="str">
+        <x:v>Components total to PS subject to limitation</x:v>
+      </x:c>
+      <x:c r="H63" s="57" t="str">
+        <x:v>Budget review / HR / Accounting</x:v>
+      </x:c>
+      <x:c r="I63" s="57" t="str">
+        <x:v>Preserve component hierarchy</x:v>
+      </x:c>
+      <x:c r="J63" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K63" s="63" t="str"/>
+      <x:c r="L63" s="63" t="str"/>
+      <x:c r="M63" s="63" t="str"/>
+      <x:c r="N63" s="57" t="str">
+        <x:v>MAP-058</x:v>
+      </x:c>
+      <x:c r="O63" s="63" t="str">
+        <x:v>DBM manual pp. 154 (PDF pp. 169)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="57" t="str">
+        <x:v>LBR Form 2B</x:v>
+      </x:c>
+      <x:c r="B64" s="57" t="str">
+        <x:v>Compliance conclusion</x:v>
+      </x:c>
+      <x:c r="C64" s="57" t="str">
+        <x:v>Total PS; waived items; adjusted PS; excess/available margin; decision evidence</x:v>
+      </x:c>
+      <x:c r="D64" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E64" s="57" t="str">
+        <x:v>Calculated PS schedule and Form 2A where applicable</x:v>
+      </x:c>
+      <x:c r="F64" s="57" t="str">
+        <x:v>Use visible helper totals instead of a hidden conclusion</x:v>
+      </x:c>
+      <x:c r="G64" s="57" t="str">
+        <x:v>Adjusted PS comparison reproduces the compliance result</x:v>
+      </x:c>
+      <x:c r="H64" s="57" t="str">
+        <x:v>Reviewing authority</x:v>
+      </x:c>
+      <x:c r="I64" s="57" t="str">
+        <x:v>Show conclusion and supporting totals together</x:v>
+      </x:c>
+      <x:c r="J64" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K64" s="63" t="str"/>
+      <x:c r="L64" s="63" t="str"/>
+      <x:c r="M64" s="63" t="str"/>
+      <x:c r="N64" s="57" t="str">
+        <x:v>MAP-059</x:v>
+      </x:c>
+      <x:c r="O64" s="63" t="str">
+        <x:v>DBM manual pp. 154 (PDF pp. 169)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="57" t="str">
+        <x:v>LBE Form 2</x:v>
+      </x:c>
+      <x:c r="B65" s="57" t="str">
+        <x:v>Authority</x:v>
+      </x:c>
+      <x:c r="C65" s="57" t="str">
+        <x:v>FY; LGU; Executive/Sanggunian office; ordinance number</x:v>
+      </x:c>
+      <x:c r="D65" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E65" s="57" t="str">
+        <x:v>Approved augmentation authority and budget calendar</x:v>
+      </x:c>
+      <x:c r="F65" s="57" t="str">
+        <x:v>Pin exact ordinance/general-provision authority</x:v>
+      </x:c>
+      <x:c r="G65" s="57" t="str">
+        <x:v>No augmentation may proceed without accepted authority</x:v>
+      </x:c>
+      <x:c r="H65" s="57" t="str">
+        <x:v>Budget / Sanggunian</x:v>
+      </x:c>
+      <x:c r="I65" s="57" t="str">
+        <x:v>Header stays with every page</x:v>
+      </x:c>
+      <x:c r="J65" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K65" s="63" t="str"/>
+      <x:c r="L65" s="63" t="str"/>
+      <x:c r="M65" s="63" t="str"/>
+      <x:c r="N65" s="57" t="str">
+        <x:v>MAP-060</x:v>
+      </x:c>
+      <x:c r="O65" s="63" t="str">
+        <x:v>DBM manual pp. 186 (PDF pp. 201)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="57" t="str">
+        <x:v>LBE Form 2</x:v>
+      </x:c>
+      <x:c r="B66" s="57" t="str">
+        <x:v>Source and use</x:v>
+      </x:c>
+      <x:c r="C66" s="57" t="str">
+        <x:v>From/to object of expenditure; expense class; amount</x:v>
+      </x:c>
+      <x:c r="D66" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E66" s="57" t="str">
+        <x:v>Posted appropriation/allotment movements</x:v>
+      </x:c>
+      <x:c r="F66" s="57" t="str">
+        <x:v>Preserve source and use as paired rows</x:v>
+      </x:c>
+      <x:c r="G66" s="57" t="str">
+        <x:v>Source total equals use total; savings and expense-class rules pass</x:v>
+      </x:c>
+      <x:c r="H66" s="57" t="str">
+        <x:v>Budget / Accounting</x:v>
+      </x:c>
+      <x:c r="I66" s="57" t="str">
+        <x:v>Side-by-side pairing and accounting format</x:v>
+      </x:c>
+      <x:c r="J66" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K66" s="63" t="str"/>
+      <x:c r="L66" s="63" t="str"/>
+      <x:c r="M66" s="63" t="str"/>
+      <x:c r="N66" s="57" t="str">
+        <x:v>MAP-061</x:v>
+      </x:c>
+      <x:c r="O66" s="63" t="str">
+        <x:v>DBM manual pp. 186 (PDF pp. 201)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="57" t="str">
+        <x:v>LBE Form 2</x:v>
+      </x:c>
+      <x:c r="B67" s="57" t="str">
+        <x:v>Certification</x:v>
+      </x:c>
+      <x:c r="C67" s="57" t="str">
+        <x:v>LBO prepared; Accountant certified; LCE/Vice-LCE approved</x:v>
+      </x:c>
+      <x:c r="D67" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E67" s="57" t="str">
+        <x:v>Wet-signature custody evidence</x:v>
+      </x:c>
+      <x:c r="F67" s="57" t="str">
+        <x:v>Use the locally confirmed authority route</x:v>
+      </x:c>
+      <x:c r="G67" s="57" t="str">
+        <x:v>Never imply digital signature</x:v>
+      </x:c>
+      <x:c r="H67" s="57" t="str">
+        <x:v>Budget / Accounting / approving authority</x:v>
+      </x:c>
+      <x:c r="I67" s="57" t="str">
+        <x:v>Preserve totals and signature space</x:v>
+      </x:c>
+      <x:c r="J67" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K67" s="63" t="str"/>
+      <x:c r="L67" s="63" t="str"/>
+      <x:c r="M67" s="63" t="str"/>
+      <x:c r="N67" s="57" t="str">
+        <x:v>MAP-062</x:v>
+      </x:c>
+      <x:c r="O67" s="63" t="str">
+        <x:v>DBM manual pp. 186 (PDF pp. 201)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="57" t="str">
+        <x:v>LBE Form 3</x:v>
+      </x:c>
+      <x:c r="B68" s="57" t="str">
+        <x:v>Adjusted receipt rows</x:v>
+      </x:c>
+      <x:c r="C68" s="57" t="str">
+        <x:v>Income source/classification; preceding-year amount; non-recurring adjustment; adjusted estimate</x:v>
+      </x:c>
+      <x:c r="D68" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E68" s="57" t="str">
+        <x:v>Posted prior-year receipts and reenactment decisions</x:v>
+      </x:c>
+      <x:c r="F68" s="57" t="str">
+        <x:v>Map accepted income classifications</x:v>
+      </x:c>
+      <x:c r="G68" s="57" t="str">
+        <x:v>Adjusted estimate equals preceding-year amount less adjustment</x:v>
+      </x:c>
+      <x:c r="H68" s="57" t="str">
+        <x:v>Treasury / Budget / Accounting</x:v>
+      </x:c>
+      <x:c r="I68" s="57" t="str">
+        <x:v>Repeat headings and income hierarchy</x:v>
+      </x:c>
+      <x:c r="J68" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K68" s="63" t="str"/>
+      <x:c r="L68" s="63" t="str"/>
+      <x:c r="M68" s="63" t="str"/>
+      <x:c r="N68" s="57" t="str">
+        <x:v>MAP-063</x:v>
+      </x:c>
+      <x:c r="O68" s="63" t="str">
+        <x:v>DBM manual pp. 187–188 (PDF pp. 202–203)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="57" t="str">
+        <x:v>LBE Form 3</x:v>
+      </x:c>
+      <x:c r="B69" s="57" t="str">
+        <x:v>Totals and certification</x:v>
+      </x:c>
+      <x:c r="C69" s="57" t="str">
+        <x:v>Regular-income subtotals; adjusted total; prepared/certified/approved route</x:v>
+      </x:c>
+      <x:c r="D69" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E69" s="57" t="str">
+        <x:v>Adjusted receipts program and wet-signature evidence</x:v>
+      </x:c>
+      <x:c r="F69" s="57" t="str">
+        <x:v>Pin exact reenactment period and source</x:v>
+      </x:c>
+      <x:c r="G69" s="57" t="str">
+        <x:v>All section totals cross-foot</x:v>
+      </x:c>
+      <x:c r="H69" s="57" t="str">
+        <x:v>Treasury / Budget / Accounting / LCE</x:v>
+      </x:c>
+      <x:c r="I69" s="57" t="str">
+        <x:v>Accounting format; signature space</x:v>
+      </x:c>
+      <x:c r="J69" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K69" s="63" t="str"/>
+      <x:c r="L69" s="63" t="str"/>
+      <x:c r="M69" s="63" t="str"/>
+      <x:c r="N69" s="57" t="str">
+        <x:v>MAP-064</x:v>
+      </x:c>
+      <x:c r="O69" s="63" t="str">
+        <x:v>DBM manual pp. 187–188 (PDF pp. 202–203)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="57" t="str">
+        <x:v>LBE Form 4</x:v>
+      </x:c>
+      <x:c r="B70" s="57" t="str">
+        <x:v>Department expenditure program</x:v>
+      </x:c>
+      <x:c r="C70" s="57" t="str">
+        <x:v>Department; mandate; vision; mission; outcome; expense-class/object rows</x:v>
+      </x:c>
+      <x:c r="D70" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E70" s="57" t="str">
+        <x:v>Preceding-year appropriation and department profile</x:v>
+      </x:c>
+      <x:c r="F70" s="57" t="str">
+        <x:v>Map only legally reenactable expenditure scope</x:v>
+      </x:c>
+      <x:c r="G70" s="57" t="str">
+        <x:v>Every included item has source authority</x:v>
+      </x:c>
+      <x:c r="H70" s="57" t="str">
+        <x:v>Department / Budget</x:v>
+      </x:c>
+      <x:c r="I70" s="57" t="str">
+        <x:v>Repeat identity and headings</x:v>
+      </x:c>
+      <x:c r="J70" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K70" s="63" t="str"/>
+      <x:c r="L70" s="63" t="str"/>
+      <x:c r="M70" s="63" t="str"/>
+      <x:c r="N70" s="57" t="str">
+        <x:v>MAP-065</x:v>
+      </x:c>
+      <x:c r="O70" s="63" t="str">
+        <x:v>DBM manual pp. 189–190 (PDF pp. 204–205)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="57" t="str">
+        <x:v>LBE Form 4</x:v>
+      </x:c>
+      <x:c r="B71" s="57" t="str">
+        <x:v>Adjustment and total</x:v>
+      </x:c>
+      <x:c r="C71" s="57" t="str">
+        <x:v>Preceding appropriation; essential-operating adjustment; adjusted appropriation; certification</x:v>
+      </x:c>
+      <x:c r="D71" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E71" s="57" t="str">
+        <x:v>Reenactment adjustments and authority evidence</x:v>
+      </x:c>
+      <x:c r="F71" s="57" t="str">
+        <x:v>Keep exclusions and essential-expense basis visible</x:v>
+      </x:c>
+      <x:c r="G71" s="57" t="str">
+        <x:v>Adjusted appropriation equals source plus/minus approved adjustment</x:v>
+      </x:c>
+      <x:c r="H71" s="57" t="str">
+        <x:v>Budget / Accounting / LCE</x:v>
+      </x:c>
+      <x:c r="I71" s="57" t="str">
+        <x:v>Accounting format and signature space</x:v>
+      </x:c>
+      <x:c r="J71" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K71" s="63" t="str"/>
+      <x:c r="L71" s="63" t="str"/>
+      <x:c r="M71" s="63" t="str"/>
+      <x:c r="N71" s="57" t="str">
+        <x:v>MAP-066</x:v>
+      </x:c>
+      <x:c r="O71" s="63" t="str">
+        <x:v>DBM manual pp. 189–190 (PDF pp. 204–205)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="57" t="str">
+        <x:v>LBE Form 5</x:v>
+      </x:c>
+      <x:c r="B72" s="57" t="str">
+        <x:v>Summary targets</x:v>
+      </x:c>
+      <x:c r="C72" s="57" t="str">
+        <x:v>LGU; department; MFO; PPA; total cost; indicator; prior accomplishment; physical target; remarks</x:v>
+      </x:c>
+      <x:c r="D72" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E72" s="57" t="str">
+        <x:v>Approved performance plan and budget</x:v>
+      </x:c>
+      <x:c r="F72" s="57" t="str">
+        <x:v>One row per PPA/indicator with pinned source</x:v>
+      </x:c>
+      <x:c r="G72" s="57" t="str">
+        <x:v>Total cost and targets reconcile to detailed form</x:v>
+      </x:c>
+      <x:c r="H72" s="57" t="str">
+        <x:v>LPDO / Budget / Treasury</x:v>
+      </x:c>
+      <x:c r="I72" s="57" t="str">
+        <x:v>Repeat headings; readable indicators</x:v>
+      </x:c>
+      <x:c r="J72" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K72" s="63" t="str"/>
+      <x:c r="L72" s="63" t="str"/>
+      <x:c r="M72" s="63" t="str"/>
+      <x:c r="N72" s="57" t="str">
+        <x:v>MAP-067</x:v>
+      </x:c>
+      <x:c r="O72" s="63" t="str">
+        <x:v>DBM manual pp. 191–192 (PDF pp. 206–207)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="57" t="str">
+        <x:v>LBE Form 5</x:v>
+      </x:c>
+      <x:c r="B73" s="57" t="str">
+        <x:v>Certification</x:v>
+      </x:c>
+      <x:c r="C73" s="57" t="str">
+        <x:v>Prepared by LPDO/LBO/Treasurer; approved by LCE</x:v>
+      </x:c>
+      <x:c r="D73" s="57" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E73" s="57" t="str">
+        <x:v>Wet-signature custody evidence</x:v>
+      </x:c>
+      <x:c r="F73" s="57" t="str">
+        <x:v>Use accepted local committee route</x:v>
+      </x:c>
+      <x:c r="G73" s="57" t="str">
+        <x:v>Never imply digital signature</x:v>
+      </x:c>
+      <x:c r="H73" s="57" t="str">
+        <x:v>LFC / LCE</x:v>
+      </x:c>
+      <x:c r="I73" s="57" t="str">
+        <x:v>Preserve signature space</x:v>
+      </x:c>
+      <x:c r="J73" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K73" s="63" t="str"/>
+      <x:c r="L73" s="63" t="str"/>
+      <x:c r="M73" s="63" t="str"/>
+      <x:c r="N73" s="57" t="str">
+        <x:v>MAP-068</x:v>
+      </x:c>
+      <x:c r="O73" s="63" t="str">
+        <x:v>DBM manual pp. 191–192 (PDF pp. 206–207)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="57" t="str">
+        <x:v>LBE Form 5A</x:v>
+      </x:c>
+      <x:c r="B74" s="57" t="str">
+        <x:v>Detailed quarterly targets</x:v>
+      </x:c>
+      <x:c r="C74" s="57" t="str">
+        <x:v>PPA/performance indicator; quarterly financial allocation; quarterly physical target</x:v>
+      </x:c>
+      <x:c r="D74" s="57" t="str">
+        <x:v>Repeating</x:v>
+      </x:c>
+      <x:c r="E74" s="57" t="str">
+        <x:v>Approved performance and allotment plan</x:v>
+      </x:c>
+      <x:c r="F74" s="57" t="str">
+        <x:v>Pin MFO/PPA/indicator and quarter basis</x:v>
+      </x:c>
+      <x:c r="G74" s="57" t="str">
+        <x:v>Quarterly allocations/targets reconcile to annual summary</x:v>
+      </x:c>
+      <x:c r="H74" s="57" t="str">
+        <x:v>Department / Budget</x:v>
+      </x:c>
+      <x:c r="I74" s="57" t="str">
+        <x:v>Quarter headings remain readable</x:v>
+      </x:c>
+      <x:c r="J74" s="63" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K74" s="63" t="str"/>
+      <x:c r="L74" s="63" t="str"/>
+      <x:c r="M74" s="63" t="str"/>
+      <x:c r="N74" s="57" t="str">
+        <x:v>MAP-069</x:v>
+      </x:c>
+      <x:c r="O74" s="63" t="str">
+        <x:v>DBM manual pp. 193 (PDF pp. 208)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="58" t="str">
+        <x:v>LBE Form 5A</x:v>
+      </x:c>
+      <x:c r="B75" s="58" t="str">
+        <x:v>Certification</x:v>
+      </x:c>
+      <x:c r="C75" s="58" t="str">
+        <x:v>LGU; department; MFO; Department Head prepared; LCE approved</x:v>
+      </x:c>
+      <x:c r="D75" s="58" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E75" s="58" t="str">
+        <x:v>Wet-signature custody evidence</x:v>
+      </x:c>
+      <x:c r="F75" s="58" t="str">
+        <x:v>Use accepted local route</x:v>
+      </x:c>
+      <x:c r="G75" s="58" t="str">
+        <x:v>Never imply digital signature</x:v>
+      </x:c>
+      <x:c r="H75" s="58" t="str">
+        <x:v>Department Head / LCE</x:v>
+      </x:c>
+      <x:c r="I75" s="58" t="str">
+        <x:v>Preserve identity and signature space</x:v>
+      </x:c>
+      <x:c r="J75" s="64" t="str">
+        <x:v>Starter - verify</x:v>
+      </x:c>
+      <x:c r="K75" s="64" t="str"/>
+      <x:c r="L75" s="64" t="str"/>
+      <x:c r="M75" s="64" t="str"/>
+      <x:c r="N75" s="58" t="str">
+        <x:v>MAP-070</x:v>
+      </x:c>
+      <x:c r="O75" s="64" t="str">
+        <x:v>DBM manual pp. 193 (PDF pp. 208)</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="J6:J30">
+  <x:conditionalFormatting sqref="J6:J75">
     <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Accepted"/>
     <x:cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="Pass"/>
     <x:cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="Ready"/>
@@ -5189,16 +7288,16 @@
     <x:cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="Fail"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="D6:D30">
+    <x:dataValidation type="list" sqref="D6:D75">
       <x:formula1>"Required,Optional,Conditional,Repeating"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J6:J30">
+    <x:dataValidation type="list" sqref="J6:J75">
       <x:formula1>"Starter - verify,Mapped - review,Trial passed,Accepted - local,Not applicable"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d490321211d40af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra138322adbaa4501"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5772,7 +7871,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bfcc99a1e34465f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc825ae5a50944b71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6237,7 +8336,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ccd3b0c28a24b67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76070f07e9814815"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6751,7 +8850,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf1d9d13beaf4cf5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R046151a214494c36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7085,7 +9184,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fc2b26a753c45ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81c9ebf866204844"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8172,7 +10271,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re786fbcabb554579"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R881a7f7f52b14245"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>